<commit_message>
Add current state analysis
</commit_message>
<xml_diff>
--- a/Annotation_Main/Main4/Main4_Katja.xlsx
+++ b/Annotation_Main/Main4/Main4_Katja.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11012"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11012"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/katja/Dropbox/Doktorat/ParlaMint/Sentiment_annotation-speeches/Annotation_Main/Main4/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9A5503C-8567-C644-8751-C199049EBEAA}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E274172-01A4-D940-B70F-281094C30E7F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="413">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="503" uniqueCount="442">
   <si>
     <t>ID</t>
   </si>
@@ -1259,6 +1259,93 @@
   </si>
   <si>
     <t>Negative</t>
+  </si>
+  <si>
+    <t>First two sentences seem to be positive, however, the speaker then outlines several negative points in the current state of affairs and ends with relatively charged questions. However, it could also be Negative, as the first part could potentially be sarcastic</t>
+  </si>
+  <si>
+    <t>Speaker presents arguments on why the proposal of the Committee is not suitable and why the governmental proposal should be supported. He outlines the negtive consequences that can occur should they support the Committee proposal.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">At the end there is a slight negative connotation, but the overall tone of the speech is positive, albeit a bit weak. </t>
+  </si>
+  <si>
+    <t>The speaker details problems and possible solutions on the systemic corruption. The topic is obviously negative, but it is hard to detect the sentiment in the speech itself, as it seems relatively negative (though a bit weak), and at the same time, a bit neutral (speaker offers no position, no explicit proposal, just "what can be done").   It could be just directly Negative (but again, a bit weak).</t>
+  </si>
+  <si>
+    <t>Uf, the speech is defensive and at beginning and end accompanied with pretty harsh (and sarcastic) words. The middle is detailing facts (as per the speaker) and is relatively neutral. However, to me, the overall speech still seems very negative, but could maybe also be M_Negative.</t>
+  </si>
+  <si>
+    <t>Speaker presenting and explaining the bill. I do not sense explicit speaker position or sentiment, mostly as we cannot discern from the text, if the speaker belongs to the Government or not. So due to the above, I would say this is relatively neutral.</t>
+  </si>
+  <si>
+    <t>Last sentence is positive, but as seems several times before, the majority of the speech is highly negative.</t>
+  </si>
+  <si>
+    <t>The speech is overall very positive, but there are also some very negative remarks weaved into it. Therefore I cannot fully say this is only positive. However, should we interpret the negative remarks as just state-of-affairs that need to be corrected, it could also be Positive.</t>
+  </si>
+  <si>
+    <t>While in the first sentence of this speech the speaker explicitly expresses agreement with the proposal, he also pinpoints the fact that it is meant to be in favour of the banks and then goes off to argue for this position, where the speech is negative. I could also maybe see this as M_Negative, should the first part be deemed positive (which for me it isn't, but it is open to interpretation as we lack sufficient context in the first part).</t>
+  </si>
+  <si>
+    <t>I would say this has some negative connotations, but it could also be Negative.</t>
+  </si>
+  <si>
+    <t>Veryyyy sarcastic.</t>
+  </si>
+  <si>
+    <t>Speaker outlines (negative) reasons why the proposal should not be supported (or rather, why they will not support it). The tone is negative, but a bit weak. Could also be M_Negative.</t>
+  </si>
+  <si>
+    <t>Could also be M_Positive, however to me the negative tone prevails overall.</t>
+  </si>
+  <si>
+    <t>Could just as well be M_Negative, or just P_Neutral</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Could also be M_Negative. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Encoding error, two speeches as once. Interpreting just the second one (Mag. Bojan Babič: …), </t>
+  </si>
+  <si>
+    <t xml:space="preserve">In terms of sentiment, I would say that this is a very mixed speech, as it outlines problems and difficulties in the case of copyright acts. I would say it could also be M_Positive. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mixed sentiment, as the speaker acknowledges the importance of the discussion around the topic, but emphasises the (negative) current state of affairs and uses some relatively harsh negative words (e.g. sramota). </t>
+  </si>
+  <si>
+    <t>Could also be N_Neutral</t>
+  </si>
+  <si>
+    <t>Maybe a bit weak, but still consistently negative.</t>
+  </si>
+  <si>
+    <t>Not a lot of context, but with the choice of words, I would say highly sarcastic.</t>
+  </si>
+  <si>
+    <t>Again, missing context, but with the quotations, I believe this to have negative connotations.</t>
+  </si>
+  <si>
+    <t>Either M_Negative or directly Negative (with a weak start and then explicitly negative in the second part of the speech).</t>
+  </si>
+  <si>
+    <t>Either M_Negative or directly Negative.  The strong words, especially in the second part of the speech to me seem pretty Negative.</t>
+  </si>
+  <si>
+    <t>Negative topic, but also sarcastic and negative remarks at the end.</t>
+  </si>
+  <si>
+    <t>The speaker calls for support of their (in their opinion) very good proposal, but the topic and the choice of words in the beginning are negative. Would have a hard time saying this is purely Positive.</t>
+  </si>
+  <si>
+    <t>Weak, but still negative.</t>
+  </si>
+  <si>
+    <t>Could also be N_Neutral, not sure abut the connotation in the first sentence of the speech.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accusatory "questions" </t>
   </si>
 </sst>
 </file>
@@ -1280,12 +1367,24 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="3">
@@ -1326,7 +1425,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -1340,6 +1439,14 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1648,7 +1755,7 @@
     <col min="1" max="1" width="39.1640625" hidden="1" customWidth="1"/>
     <col min="2" max="2" width="124.6640625" style="3" customWidth="1"/>
     <col min="3" max="3" width="27" customWidth="1"/>
-    <col min="4" max="4" width="22.83203125" customWidth="1"/>
+    <col min="4" max="4" width="22.83203125" style="3" customWidth="1"/>
     <col min="6" max="6" width="0" hidden="1" customWidth="1"/>
     <col min="7" max="7" width="18.5" hidden="1" customWidth="1"/>
   </cols>
@@ -1663,7 +1770,7 @@
       <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
@@ -1700,6 +1807,15 @@
       <c r="B3" s="3" t="s">
         <v>9</v>
       </c>
+      <c r="C3" t="s">
+        <v>411</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>413</v>
+      </c>
+      <c r="E3" t="b">
+        <v>1</v>
+      </c>
       <c r="F3" t="b">
         <v>0</v>
       </c>
@@ -1714,6 +1830,9 @@
       <c r="B4" s="3" t="s">
         <v>11</v>
       </c>
+      <c r="C4" t="s">
+        <v>408</v>
+      </c>
       <c r="F4" t="b">
         <v>1</v>
       </c>
@@ -1721,12 +1840,18 @@
         <v>409</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="112" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" ht="160" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>12</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>13</v>
+      </c>
+      <c r="C5" t="s">
+        <v>412</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>414</v>
       </c>
       <c r="F5" t="b">
         <v>0</v>
@@ -1742,6 +1867,12 @@
       <c r="B6" s="3" t="s">
         <v>15</v>
       </c>
+      <c r="C6" t="s">
+        <v>407</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>415</v>
+      </c>
       <c r="F6" t="b">
         <v>0</v>
       </c>
@@ -1756,6 +1887,9 @@
       <c r="B7" s="3" t="s">
         <v>17</v>
       </c>
+      <c r="C7" t="s">
+        <v>412</v>
+      </c>
       <c r="F7" t="b">
         <v>0</v>
       </c>
@@ -1770,6 +1904,9 @@
       <c r="B8" s="3" t="s">
         <v>19</v>
       </c>
+      <c r="C8" t="s">
+        <v>412</v>
+      </c>
       <c r="F8" t="b">
         <v>0</v>
       </c>
@@ -1778,8 +1915,17 @@
       <c r="A9" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="5" t="s">
         <v>21</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>411</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>416</v>
+      </c>
+      <c r="E9" s="6" t="b">
+        <v>1</v>
       </c>
       <c r="F9" t="b">
         <v>0</v>
@@ -1792,16 +1938,28 @@
       <c r="B10" s="3" t="s">
         <v>23</v>
       </c>
+      <c r="C10" t="s">
+        <v>408</v>
+      </c>
       <c r="F10" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="160" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" ht="176" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>24</v>
       </c>
-      <c r="B11" s="3" t="s">
+      <c r="B11" s="5" t="s">
         <v>25</v>
+      </c>
+      <c r="C11" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>417</v>
+      </c>
+      <c r="E11" s="6" t="b">
+        <v>1</v>
       </c>
       <c r="F11" t="b">
         <v>0</v>
@@ -1811,8 +1969,17 @@
       <c r="A12" t="s">
         <v>26</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="5" t="s">
         <v>27</v>
+      </c>
+      <c r="C12" s="6" t="s">
+        <v>408</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>418</v>
+      </c>
+      <c r="E12" s="6" t="b">
+        <v>1</v>
       </c>
       <c r="F12" t="b">
         <v>0</v>
@@ -1825,6 +1992,12 @@
       <c r="B13" s="3" t="s">
         <v>29</v>
       </c>
+      <c r="C13" t="s">
+        <v>412</v>
+      </c>
+      <c r="D13" s="3" t="s">
+        <v>419</v>
+      </c>
       <c r="F13" t="b">
         <v>0</v>
       </c>
@@ -1836,6 +2009,9 @@
       <c r="B14" s="3" t="s">
         <v>31</v>
       </c>
+      <c r="C14" t="s">
+        <v>408</v>
+      </c>
       <c r="F14" t="b">
         <v>1</v>
       </c>
@@ -1847,6 +2023,9 @@
       <c r="B15" s="3" t="s">
         <v>33</v>
       </c>
+      <c r="C15" t="s">
+        <v>412</v>
+      </c>
       <c r="F15" t="b">
         <v>0</v>
       </c>
@@ -1858,6 +2037,12 @@
       <c r="B16" s="3" t="s">
         <v>35</v>
       </c>
+      <c r="C16" t="s">
+        <v>410</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>420</v>
+      </c>
       <c r="F16" t="b">
         <v>0</v>
       </c>
@@ -1869,6 +2054,15 @@
       <c r="B17" s="3" t="s">
         <v>37</v>
       </c>
+      <c r="C17" t="s">
+        <v>412</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>421</v>
+      </c>
+      <c r="E17" t="b">
+        <v>1</v>
+      </c>
       <c r="F17" t="b">
         <v>0</v>
       </c>
@@ -1877,8 +2071,17 @@
       <c r="A18" t="s">
         <v>38</v>
       </c>
-      <c r="B18" s="3" t="s">
+      <c r="B18" s="5" t="s">
         <v>39</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>409</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>422</v>
+      </c>
+      <c r="E18" s="6" t="b">
+        <v>1</v>
       </c>
       <c r="F18" t="b">
         <v>1</v>
@@ -1891,6 +2094,12 @@
       <c r="B19" s="3" t="s">
         <v>41</v>
       </c>
+      <c r="C19" t="s">
+        <v>412</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>423</v>
+      </c>
       <c r="F19" t="b">
         <v>0</v>
       </c>
@@ -1902,6 +2111,9 @@
       <c r="B20" s="3" t="s">
         <v>43</v>
       </c>
+      <c r="C20" t="s">
+        <v>412</v>
+      </c>
       <c r="F20" t="b">
         <v>0</v>
       </c>
@@ -1910,8 +2122,17 @@
       <c r="A21" t="s">
         <v>44</v>
       </c>
-      <c r="B21" s="3" t="s">
+      <c r="B21" s="5" t="s">
         <v>45</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>424</v>
+      </c>
+      <c r="E21" s="6" t="b">
+        <v>1</v>
       </c>
       <c r="F21" t="b">
         <v>0</v>
@@ -1924,6 +2145,9 @@
       <c r="B22" s="3" t="s">
         <v>47</v>
       </c>
+      <c r="C22" t="s">
+        <v>412</v>
+      </c>
       <c r="F22" t="b">
         <v>0</v>
       </c>
@@ -1932,8 +2156,17 @@
       <c r="A23" t="s">
         <v>48</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B23" s="5" t="s">
         <v>49</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>411</v>
+      </c>
+      <c r="D23" s="5" t="s">
+        <v>425</v>
+      </c>
+      <c r="E23" s="6" t="b">
+        <v>1</v>
       </c>
       <c r="F23" t="b">
         <v>0</v>
@@ -1946,16 +2179,31 @@
       <c r="B24" s="3" t="s">
         <v>51</v>
       </c>
+      <c r="C24" t="s">
+        <v>410</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>427</v>
+      </c>
       <c r="F24" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:6" ht="48" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>52</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>53</v>
+      </c>
+      <c r="C25" t="s">
+        <v>409</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>426</v>
+      </c>
+      <c r="E25" t="b">
+        <v>1</v>
       </c>
       <c r="F25" t="b">
         <v>1</v>
@@ -1965,9 +2213,14 @@
       <c r="A26" t="s">
         <v>54</v>
       </c>
-      <c r="B26" s="3" t="s">
+      <c r="B26" s="7" t="s">
         <v>55</v>
       </c>
+      <c r="C26" s="8"/>
+      <c r="D26" s="7" t="s">
+        <v>428</v>
+      </c>
+      <c r="E26" s="8"/>
       <c r="F26" t="b">
         <v>1</v>
       </c>
@@ -1979,6 +2232,9 @@
       <c r="B27" s="3" t="s">
         <v>57</v>
       </c>
+      <c r="C27" t="s">
+        <v>408</v>
+      </c>
       <c r="F27" t="b">
         <v>0</v>
       </c>
@@ -1990,6 +2246,9 @@
       <c r="B28" s="3" t="s">
         <v>59</v>
       </c>
+      <c r="C28" t="s">
+        <v>408</v>
+      </c>
       <c r="F28" t="b">
         <v>1</v>
       </c>
@@ -1998,8 +2257,17 @@
       <c r="A29" t="s">
         <v>60</v>
       </c>
-      <c r="B29" s="3" t="s">
+      <c r="B29" s="5" t="s">
         <v>61</v>
+      </c>
+      <c r="C29" s="6" t="s">
+        <v>411</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>429</v>
+      </c>
+      <c r="E29" s="6" t="b">
+        <v>1</v>
       </c>
       <c r="F29" t="b">
         <v>0</v>
@@ -2012,6 +2280,9 @@
       <c r="B30" s="3" t="s">
         <v>63</v>
       </c>
+      <c r="C30" t="s">
+        <v>408</v>
+      </c>
       <c r="F30" t="b">
         <v>0</v>
       </c>
@@ -2023,6 +2294,12 @@
       <c r="B31" s="3" t="s">
         <v>65</v>
       </c>
+      <c r="C31" t="s">
+        <v>411</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>430</v>
+      </c>
       <c r="F31" t="b">
         <v>0</v>
       </c>
@@ -2031,8 +2308,17 @@
       <c r="A32" t="s">
         <v>66</v>
       </c>
-      <c r="B32" s="3" t="s">
+      <c r="B32" s="5" t="s">
         <v>67</v>
+      </c>
+      <c r="C32" s="6" t="s">
+        <v>408</v>
+      </c>
+      <c r="D32" s="5" t="s">
+        <v>431</v>
+      </c>
+      <c r="E32" t="b">
+        <v>1</v>
       </c>
       <c r="F32" t="b">
         <v>1</v>
@@ -2045,6 +2331,9 @@
       <c r="B33" s="3" t="s">
         <v>69</v>
       </c>
+      <c r="C33" t="s">
+        <v>412</v>
+      </c>
       <c r="F33" t="b">
         <v>0</v>
       </c>
@@ -2056,6 +2345,9 @@
       <c r="B34" s="3" t="s">
         <v>71</v>
       </c>
+      <c r="C34" t="s">
+        <v>408</v>
+      </c>
       <c r="F34" t="b">
         <v>1</v>
       </c>
@@ -2067,6 +2359,9 @@
       <c r="B35" s="3" t="s">
         <v>73</v>
       </c>
+      <c r="C35" t="s">
+        <v>408</v>
+      </c>
       <c r="F35" t="b">
         <v>1</v>
       </c>
@@ -2078,6 +2373,9 @@
       <c r="B36" s="3" t="s">
         <v>75</v>
       </c>
+      <c r="C36" t="s">
+        <v>412</v>
+      </c>
       <c r="F36" t="b">
         <v>0</v>
       </c>
@@ -2089,6 +2387,9 @@
       <c r="B37" s="3" t="s">
         <v>77</v>
       </c>
+      <c r="C37" t="s">
+        <v>408</v>
+      </c>
       <c r="F37" t="b">
         <v>1</v>
       </c>
@@ -2100,6 +2401,9 @@
       <c r="B38" s="3" t="s">
         <v>79</v>
       </c>
+      <c r="C38" t="s">
+        <v>408</v>
+      </c>
       <c r="F38" t="b">
         <v>1</v>
       </c>
@@ -2111,16 +2415,28 @@
       <c r="B39" s="3" t="s">
         <v>81</v>
       </c>
+      <c r="C39" t="s">
+        <v>412</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>432</v>
+      </c>
       <c r="F39" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:6" ht="48" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>82</v>
       </c>
       <c r="B40" s="3" t="s">
         <v>83</v>
+      </c>
+      <c r="C40" t="s">
+        <v>412</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>433</v>
       </c>
       <c r="F40" t="b">
         <v>0</v>
@@ -2133,16 +2449,25 @@
       <c r="B41" s="3" t="s">
         <v>85</v>
       </c>
+      <c r="C41" t="s">
+        <v>408</v>
+      </c>
       <c r="F41" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:6" ht="64" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>86</v>
       </c>
       <c r="B42" s="3" t="s">
         <v>87</v>
+      </c>
+      <c r="C42" t="s">
+        <v>409</v>
+      </c>
+      <c r="D42" s="3" t="s">
+        <v>434</v>
       </c>
       <c r="F42" t="b">
         <v>0</v>
@@ -2155,6 +2480,9 @@
       <c r="B43" s="3" t="s">
         <v>89</v>
       </c>
+      <c r="C43" t="s">
+        <v>408</v>
+      </c>
       <c r="F43" t="b">
         <v>1</v>
       </c>
@@ -2163,8 +2491,17 @@
       <c r="A44" t="s">
         <v>90</v>
       </c>
-      <c r="B44" s="3" t="s">
+      <c r="B44" s="5" t="s">
         <v>91</v>
+      </c>
+      <c r="C44" s="6" t="s">
+        <v>411</v>
+      </c>
+      <c r="D44" s="5" t="s">
+        <v>435</v>
+      </c>
+      <c r="E44" s="6" t="b">
+        <v>1</v>
       </c>
       <c r="F44" t="b">
         <v>0</v>
@@ -2177,6 +2514,9 @@
       <c r="B45" s="3" t="s">
         <v>93</v>
       </c>
+      <c r="C45" t="s">
+        <v>408</v>
+      </c>
       <c r="F45" t="b">
         <v>1</v>
       </c>
@@ -2188,6 +2528,9 @@
       <c r="B46" s="3" t="s">
         <v>95</v>
       </c>
+      <c r="C46" t="s">
+        <v>408</v>
+      </c>
       <c r="F46" t="b">
         <v>1</v>
       </c>
@@ -2199,6 +2542,9 @@
       <c r="B47" s="3" t="s">
         <v>97</v>
       </c>
+      <c r="C47" t="s">
+        <v>408</v>
+      </c>
       <c r="F47" t="b">
         <v>1</v>
       </c>
@@ -2210,6 +2556,9 @@
       <c r="B48" s="3" t="s">
         <v>99</v>
       </c>
+      <c r="C48" t="s">
+        <v>408</v>
+      </c>
       <c r="F48" t="b">
         <v>1</v>
       </c>
@@ -2221,6 +2570,9 @@
       <c r="B49" s="3" t="s">
         <v>101</v>
       </c>
+      <c r="C49" t="s">
+        <v>408</v>
+      </c>
       <c r="F49" t="b">
         <v>1</v>
       </c>
@@ -2232,6 +2584,9 @@
       <c r="B50" s="3" t="s">
         <v>103</v>
       </c>
+      <c r="C50" t="s">
+        <v>412</v>
+      </c>
       <c r="F50" t="b">
         <v>0</v>
       </c>
@@ -2243,6 +2598,15 @@
       <c r="B51" s="3" t="s">
         <v>105</v>
       </c>
+      <c r="C51" t="s">
+        <v>412</v>
+      </c>
+      <c r="D51" s="3" t="s">
+        <v>436</v>
+      </c>
+      <c r="E51" t="b">
+        <v>1</v>
+      </c>
       <c r="F51" t="b">
         <v>0</v>
       </c>
@@ -2254,6 +2618,12 @@
       <c r="B52" s="3" t="s">
         <v>107</v>
       </c>
+      <c r="C52" t="s">
+        <v>412</v>
+      </c>
+      <c r="D52" s="3" t="s">
+        <v>437</v>
+      </c>
       <c r="F52" t="b">
         <v>0</v>
       </c>
@@ -2265,6 +2635,9 @@
       <c r="B53" s="3" t="s">
         <v>109</v>
       </c>
+      <c r="C53" t="s">
+        <v>408</v>
+      </c>
       <c r="F53" t="b">
         <v>1</v>
       </c>
@@ -2276,6 +2649,9 @@
       <c r="B54" s="3" t="s">
         <v>111</v>
       </c>
+      <c r="C54" t="s">
+        <v>408</v>
+      </c>
       <c r="F54" t="b">
         <v>1</v>
       </c>
@@ -2287,16 +2663,25 @@
       <c r="B55" s="3" t="s">
         <v>113</v>
       </c>
+      <c r="C55" t="s">
+        <v>408</v>
+      </c>
       <c r="F55" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:6" ht="64" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:6" ht="128" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>114</v>
       </c>
       <c r="B56" s="3" t="s">
         <v>115</v>
+      </c>
+      <c r="C56" t="s">
+        <v>410</v>
+      </c>
+      <c r="D56" s="3" t="s">
+        <v>438</v>
       </c>
       <c r="F56" t="b">
         <v>0</v>
@@ -2309,6 +2694,12 @@
       <c r="B57" s="3" t="s">
         <v>117</v>
       </c>
+      <c r="C57" t="s">
+        <v>412</v>
+      </c>
+      <c r="D57" s="3" t="s">
+        <v>439</v>
+      </c>
       <c r="F57" t="b">
         <v>0</v>
       </c>
@@ -2320,6 +2711,9 @@
       <c r="B58" s="3" t="s">
         <v>119</v>
       </c>
+      <c r="C58" t="s">
+        <v>408</v>
+      </c>
       <c r="F58" t="b">
         <v>1</v>
       </c>
@@ -2331,6 +2725,9 @@
       <c r="B59" s="3" t="s">
         <v>121</v>
       </c>
+      <c r="C59" t="s">
+        <v>408</v>
+      </c>
       <c r="F59" t="b">
         <v>1</v>
       </c>
@@ -2342,6 +2739,9 @@
       <c r="B60" s="3" t="s">
         <v>123</v>
       </c>
+      <c r="C60" t="s">
+        <v>408</v>
+      </c>
       <c r="F60" t="b">
         <v>1</v>
       </c>
@@ -2353,16 +2753,28 @@
       <c r="B61" s="3" t="s">
         <v>125</v>
       </c>
+      <c r="C61" t="s">
+        <v>408</v>
+      </c>
       <c r="F61" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:6" ht="64" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>126</v>
       </c>
       <c r="B62" s="3" t="s">
         <v>127</v>
+      </c>
+      <c r="C62" t="s">
+        <v>408</v>
+      </c>
+      <c r="D62" s="3" t="s">
+        <v>440</v>
+      </c>
+      <c r="E62" t="b">
+        <v>1</v>
       </c>
       <c r="F62" t="b">
         <v>1</v>
@@ -2375,6 +2787,12 @@
       <c r="B63" s="3" t="s">
         <v>129</v>
       </c>
+      <c r="C63" t="s">
+        <v>412</v>
+      </c>
+      <c r="D63" s="3" t="s">
+        <v>441</v>
+      </c>
       <c r="F63" t="b">
         <v>0</v>
       </c>
@@ -3899,7 +4317,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C1:C1048576" xr:uid="{0454D887-4936-5541-AB4A-96E9F5E46179}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C1:C1048576" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>$G$2:$G$7</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Calculate ACC for non-procedural speeches
</commit_message>
<xml_diff>
--- a/Annotation_Main/Main4/Main4_Katja.xlsx
+++ b/Annotation_Main/Main4/Main4_Katja.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/katja/Dropbox/Doktorat/ParlaMint/Sentiment_annotation-speeches/Annotation_Main/Main4/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3E274172-01A4-D940-B70F-281094C30E7F}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEBCA7C7-0E5F-AF4D-AEE2-45B9BD62C7DC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="503" uniqueCount="442">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="618" uniqueCount="466">
   <si>
     <t>ID</t>
   </si>
@@ -1346,6 +1346,78 @@
   </si>
   <si>
     <t xml:space="preserve">Accusatory "questions" </t>
+  </si>
+  <si>
+    <t>Very mixed sentiment throughout the speech. The speaker and his PS supports the amendments, but at the same time consistently brings out several negative points about the procedure in which the amendment was proposed. Overall, while there is support, the tone is to me leaning slightly more to negative, but could also be M_Positive</t>
+  </si>
+  <si>
+    <t xml:space="preserve">To me this feels slightly defensive, and while there are some positive points in the speech. </t>
+  </si>
+  <si>
+    <t>Just a statement but with slight negative connotation.</t>
+  </si>
+  <si>
+    <t>Could also be Negative.</t>
+  </si>
+  <si>
+    <t>As this outlines the positive changes of the proposal, I would consider it positive, but rather weak. Could also be P_Neutral</t>
+  </si>
+  <si>
+    <t>First part is slightly less negative, even positive at certain points, and then the sentiment changes into fully negative mid speech.</t>
+  </si>
+  <si>
+    <t>Positive topic, or at least positive changes, middle part of the speech just explains the bill and speaker calls for support with a positive statement at the end. So the sentiment might be weak, but is consistently (slightly) positive .</t>
+  </si>
+  <si>
+    <t>Very confused speech and would probably consider different label, should be words not be so weirdly specific.</t>
+  </si>
+  <si>
+    <t>Hm..The speaker himself states that (presumably) this will be a positive reply. But to me this is mostly M_Positive at best, as the middle part seems defensive.</t>
+  </si>
+  <si>
+    <t>First part positive, second negative. But due to the very negative second part, this could be fully Negative.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The middle part of speech is slight less negative, maybe even neutral, as it outlines cheanges that should be in place for this proposed changes to be sucessful, so not really positive. </t>
+  </si>
+  <si>
+    <t>I don't sense a particular sentiment here. It is very procedural in nature.</t>
+  </si>
+  <si>
+    <t>First part is positive, but is very short, so this could also be Negative</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Warning </t>
+  </si>
+  <si>
+    <t>Explicit and harsh warning to the speaker.</t>
+  </si>
+  <si>
+    <t>Charged and agressive speech.</t>
+  </si>
+  <si>
+    <t>Middle part is not as negative, might even be slightly positive, but there is too much negative tone in it for me to consider it M_Negative.</t>
+  </si>
+  <si>
+    <t>Last part is slightly negtive But if we look overall, it could be Positive.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">First two sentences seem truly positive, however, the majority of the speech is so negative and at points sarcastic that I feel this is just Negative. But could also be M_Negative. </t>
+  </si>
+  <si>
+    <t>There are some points that seem slightly sarcastic/negative. But overall it s positive in tone, so maybe it can also be purely Positive</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Majority of speech positive, but in the second part the sentiment turns to negative (..."Kljub temu pa smo v  poslanski skupini ugotovili vrsto pomanjkljivosti). </t>
+  </si>
+  <si>
+    <t>Could also be P_Neutral</t>
+  </si>
+  <si>
+    <t>Seems like a warning to the speaker. Could just as well be directly Negative.</t>
+  </si>
+  <si>
+    <t>Uffff, negative (probably procedural).</t>
   </si>
 </sst>
 </file>
@@ -2804,6 +2876,15 @@
       <c r="B64" s="3" t="s">
         <v>131</v>
       </c>
+      <c r="C64" t="s">
+        <v>411</v>
+      </c>
+      <c r="D64" s="3" t="s">
+        <v>442</v>
+      </c>
+      <c r="E64" t="b">
+        <v>1</v>
+      </c>
       <c r="F64" t="b">
         <v>0</v>
       </c>
@@ -2815,6 +2896,12 @@
       <c r="B65" s="3" t="s">
         <v>133</v>
       </c>
+      <c r="C65" t="s">
+        <v>411</v>
+      </c>
+      <c r="D65" s="3" t="s">
+        <v>443</v>
+      </c>
       <c r="F65" t="b">
         <v>0</v>
       </c>
@@ -2826,16 +2913,25 @@
       <c r="B66" s="3" t="s">
         <v>135</v>
       </c>
+      <c r="C66" t="s">
+        <v>408</v>
+      </c>
       <c r="F66" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:6" ht="32" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>136</v>
       </c>
-      <c r="B67" s="3" t="s">
+      <c r="B67" s="5" t="s">
         <v>137</v>
+      </c>
+      <c r="C67" s="6" t="s">
+        <v>409</v>
+      </c>
+      <c r="D67" s="5" t="s">
+        <v>444</v>
       </c>
       <c r="F67" t="b">
         <v>0</v>
@@ -2848,6 +2944,9 @@
       <c r="B68" s="3" t="s">
         <v>139</v>
       </c>
+      <c r="C68" t="s">
+        <v>408</v>
+      </c>
       <c r="F68" t="b">
         <v>1</v>
       </c>
@@ -2859,6 +2958,9 @@
       <c r="B69" s="3" t="s">
         <v>141</v>
       </c>
+      <c r="C69" t="s">
+        <v>408</v>
+      </c>
       <c r="F69" t="b">
         <v>1</v>
       </c>
@@ -2870,6 +2972,15 @@
       <c r="B70" s="3" t="s">
         <v>143</v>
       </c>
+      <c r="C70" t="s">
+        <v>409</v>
+      </c>
+      <c r="D70" s="3" t="s">
+        <v>445</v>
+      </c>
+      <c r="E70" t="b">
+        <v>1</v>
+      </c>
       <c r="F70" t="b">
         <v>1</v>
       </c>
@@ -2878,9 +2989,14 @@
       <c r="A71" t="s">
         <v>144</v>
       </c>
-      <c r="B71" s="3" t="s">
+      <c r="B71" s="5" t="s">
         <v>145</v>
       </c>
+      <c r="C71" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="D71" s="5"/>
+      <c r="E71" s="6"/>
       <c r="F71" t="b">
         <v>0</v>
       </c>
@@ -2892,6 +3008,12 @@
       <c r="B72" s="3" t="s">
         <v>147</v>
       </c>
+      <c r="C72" t="s">
+        <v>407</v>
+      </c>
+      <c r="D72" s="3" t="s">
+        <v>446</v>
+      </c>
       <c r="F72" t="b">
         <v>0</v>
       </c>
@@ -2903,6 +3025,12 @@
       <c r="B73" s="3" t="s">
         <v>149</v>
       </c>
+      <c r="C73" t="s">
+        <v>411</v>
+      </c>
+      <c r="D73" s="3" t="s">
+        <v>447</v>
+      </c>
       <c r="F73" t="b">
         <v>0</v>
       </c>
@@ -2914,16 +3042,25 @@
       <c r="B74" s="3" t="s">
         <v>151</v>
       </c>
+      <c r="C74" t="s">
+        <v>408</v>
+      </c>
       <c r="F74" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:6" ht="128" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:6" ht="144" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>152</v>
       </c>
       <c r="B75" s="3" t="s">
         <v>153</v>
+      </c>
+      <c r="C75" t="s">
+        <v>407</v>
+      </c>
+      <c r="D75" s="3" t="s">
+        <v>448</v>
       </c>
       <c r="F75" t="b">
         <v>0</v>
@@ -2936,6 +3073,9 @@
       <c r="B76" s="3" t="s">
         <v>155</v>
       </c>
+      <c r="C76" t="s">
+        <v>408</v>
+      </c>
       <c r="F76" t="b">
         <v>1</v>
       </c>
@@ -2944,9 +3084,13 @@
       <c r="A77" t="s">
         <v>156</v>
       </c>
-      <c r="B77" s="3" t="s">
+      <c r="B77" s="5" t="s">
         <v>157</v>
       </c>
+      <c r="C77" s="6" t="s">
+        <v>409</v>
+      </c>
+      <c r="D77" s="5"/>
       <c r="F77" t="b">
         <v>0</v>
       </c>
@@ -2955,9 +3099,13 @@
       <c r="A78" t="s">
         <v>158</v>
       </c>
-      <c r="B78" s="3" t="s">
+      <c r="B78" s="5" t="s">
         <v>159</v>
       </c>
+      <c r="C78" s="6" t="s">
+        <v>408</v>
+      </c>
+      <c r="D78" s="5"/>
       <c r="F78" t="b">
         <v>1</v>
       </c>
@@ -2969,6 +3117,9 @@
       <c r="B79" s="3" t="s">
         <v>161</v>
       </c>
+      <c r="C79" t="s">
+        <v>408</v>
+      </c>
       <c r="F79" t="b">
         <v>1</v>
       </c>
@@ -2977,8 +3128,17 @@
       <c r="A80" t="s">
         <v>162</v>
       </c>
-      <c r="B80" s="3" t="s">
+      <c r="B80" s="5" t="s">
         <v>163</v>
+      </c>
+      <c r="C80" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="D80" s="5" t="s">
+        <v>449</v>
+      </c>
+      <c r="E80" s="6" t="b">
+        <v>1</v>
       </c>
       <c r="F80" t="b">
         <v>0</v>
@@ -2991,6 +3151,9 @@
       <c r="B81" s="3" t="s">
         <v>165</v>
       </c>
+      <c r="C81" t="s">
+        <v>408</v>
+      </c>
       <c r="F81" t="b">
         <v>1</v>
       </c>
@@ -3002,6 +3165,9 @@
       <c r="B82" s="3" t="s">
         <v>167</v>
       </c>
+      <c r="C82" t="s">
+        <v>408</v>
+      </c>
       <c r="F82" t="b">
         <v>1</v>
       </c>
@@ -3013,6 +3179,9 @@
       <c r="B83" s="3" t="s">
         <v>169</v>
       </c>
+      <c r="C83" t="s">
+        <v>408</v>
+      </c>
       <c r="F83" t="b">
         <v>1</v>
       </c>
@@ -3024,6 +3193,9 @@
       <c r="B84" s="3" t="s">
         <v>171</v>
       </c>
+      <c r="C84" t="s">
+        <v>412</v>
+      </c>
       <c r="F84" t="b">
         <v>0</v>
       </c>
@@ -3035,6 +3207,9 @@
       <c r="B85" s="3" t="s">
         <v>173</v>
       </c>
+      <c r="C85" t="s">
+        <v>408</v>
+      </c>
       <c r="F85" t="b">
         <v>1</v>
       </c>
@@ -3046,16 +3221,28 @@
       <c r="B86" s="3" t="s">
         <v>175</v>
       </c>
+      <c r="C86" t="s">
+        <v>408</v>
+      </c>
       <c r="F86" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="87" spans="1:6" ht="48" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:6" ht="112" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>176</v>
       </c>
-      <c r="B87" s="3" t="s">
+      <c r="B87" s="5" t="s">
         <v>177</v>
+      </c>
+      <c r="C87" s="6" t="s">
+        <v>410</v>
+      </c>
+      <c r="D87" s="5" t="s">
+        <v>450</v>
+      </c>
+      <c r="E87" s="6" t="b">
+        <v>1</v>
       </c>
       <c r="F87" t="b">
         <v>0</v>
@@ -3065,8 +3252,17 @@
       <c r="A88" t="s">
         <v>178</v>
       </c>
-      <c r="B88" s="3" t="s">
+      <c r="B88" s="5" t="s">
         <v>179</v>
+      </c>
+      <c r="C88" s="6" t="s">
+        <v>411</v>
+      </c>
+      <c r="D88" s="5" t="s">
+        <v>451</v>
+      </c>
+      <c r="E88" s="6" t="b">
+        <v>1</v>
       </c>
       <c r="F88" t="b">
         <v>0</v>
@@ -3079,6 +3275,12 @@
       <c r="B89" s="3" t="s">
         <v>181</v>
       </c>
+      <c r="C89" t="s">
+        <v>412</v>
+      </c>
+      <c r="D89" s="3" t="s">
+        <v>452</v>
+      </c>
       <c r="F89" t="b">
         <v>0</v>
       </c>
@@ -3090,6 +3292,12 @@
       <c r="B90" s="3" t="s">
         <v>183</v>
       </c>
+      <c r="C90" t="s">
+        <v>408</v>
+      </c>
+      <c r="D90" s="3" t="s">
+        <v>453</v>
+      </c>
       <c r="F90" t="b">
         <v>0</v>
       </c>
@@ -3101,6 +3309,9 @@
       <c r="B91" s="3" t="s">
         <v>185</v>
       </c>
+      <c r="C91" t="s">
+        <v>408</v>
+      </c>
       <c r="F91" t="b">
         <v>1</v>
       </c>
@@ -3112,6 +3323,9 @@
       <c r="B92" s="3" t="s">
         <v>187</v>
       </c>
+      <c r="C92" t="s">
+        <v>412</v>
+      </c>
       <c r="F92" t="b">
         <v>0</v>
       </c>
@@ -3120,9 +3334,13 @@
       <c r="A93" t="s">
         <v>188</v>
       </c>
-      <c r="B93" s="3" t="s">
+      <c r="B93" s="5" t="s">
         <v>189</v>
       </c>
+      <c r="C93" s="6" t="s">
+        <v>409</v>
+      </c>
+      <c r="D93" s="5"/>
       <c r="F93" t="b">
         <v>1</v>
       </c>
@@ -3134,6 +3352,12 @@
       <c r="B94" s="3" t="s">
         <v>191</v>
       </c>
+      <c r="C94" t="s">
+        <v>412</v>
+      </c>
+      <c r="D94" s="3" t="s">
+        <v>456</v>
+      </c>
       <c r="F94" t="b">
         <v>1</v>
       </c>
@@ -3145,6 +3369,15 @@
       <c r="B95" s="3" t="s">
         <v>193</v>
       </c>
+      <c r="C95" t="s">
+        <v>411</v>
+      </c>
+      <c r="D95" s="3" t="s">
+        <v>454</v>
+      </c>
+      <c r="E95" t="b">
+        <v>1</v>
+      </c>
       <c r="F95" t="b">
         <v>0</v>
       </c>
@@ -3156,6 +3389,9 @@
       <c r="B96" s="3" t="s">
         <v>195</v>
       </c>
+      <c r="C96" t="s">
+        <v>408</v>
+      </c>
       <c r="F96" t="b">
         <v>1</v>
       </c>
@@ -3167,6 +3403,12 @@
       <c r="B97" s="3" t="s">
         <v>197</v>
       </c>
+      <c r="C97" t="s">
+        <v>412</v>
+      </c>
+      <c r="D97" s="3" t="s">
+        <v>455</v>
+      </c>
       <c r="F97" t="b">
         <v>1</v>
       </c>
@@ -3178,6 +3420,9 @@
       <c r="B98" s="3" t="s">
         <v>199</v>
       </c>
+      <c r="C98" t="s">
+        <v>412</v>
+      </c>
       <c r="F98" t="b">
         <v>0</v>
       </c>
@@ -3189,6 +3434,9 @@
       <c r="B99" s="3" t="s">
         <v>201</v>
       </c>
+      <c r="C99" t="s">
+        <v>412</v>
+      </c>
       <c r="F99" t="b">
         <v>0</v>
       </c>
@@ -3200,6 +3448,9 @@
       <c r="B100" s="3" t="s">
         <v>203</v>
       </c>
+      <c r="C100" t="s">
+        <v>408</v>
+      </c>
       <c r="F100" t="b">
         <v>1</v>
       </c>
@@ -3211,6 +3462,9 @@
       <c r="B101" s="3" t="s">
         <v>205</v>
       </c>
+      <c r="C101" t="s">
+        <v>408</v>
+      </c>
       <c r="F101" t="b">
         <v>1</v>
       </c>
@@ -3222,6 +3476,9 @@
       <c r="B102" s="3" t="s">
         <v>207</v>
       </c>
+      <c r="C102" t="s">
+        <v>412</v>
+      </c>
       <c r="F102" t="b">
         <v>0</v>
       </c>
@@ -3233,6 +3490,9 @@
       <c r="B103" s="3" t="s">
         <v>209</v>
       </c>
+      <c r="C103" t="s">
+        <v>412</v>
+      </c>
       <c r="F103" t="b">
         <v>0</v>
       </c>
@@ -3244,6 +3504,9 @@
       <c r="B104" s="3" t="s">
         <v>211</v>
       </c>
+      <c r="C104" t="s">
+        <v>408</v>
+      </c>
       <c r="F104" t="b">
         <v>1</v>
       </c>
@@ -3255,6 +3518,9 @@
       <c r="B105" s="3" t="s">
         <v>213</v>
       </c>
+      <c r="C105" t="s">
+        <v>408</v>
+      </c>
       <c r="F105" t="b">
         <v>1</v>
       </c>
@@ -3266,6 +3532,9 @@
       <c r="B106" s="3" t="s">
         <v>215</v>
       </c>
+      <c r="C106" t="s">
+        <v>412</v>
+      </c>
       <c r="F106" t="b">
         <v>0</v>
       </c>
@@ -3277,6 +3546,9 @@
       <c r="B107" s="3" t="s">
         <v>217</v>
       </c>
+      <c r="C107" t="s">
+        <v>408</v>
+      </c>
       <c r="F107" t="b">
         <v>1</v>
       </c>
@@ -3288,16 +3560,31 @@
       <c r="B108" s="3" t="s">
         <v>219</v>
       </c>
+      <c r="C108" t="s">
+        <v>412</v>
+      </c>
+      <c r="D108" s="3" t="s">
+        <v>457</v>
+      </c>
       <c r="F108" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:6" ht="48" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:6" ht="96" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>220</v>
       </c>
-      <c r="B109" s="3" t="s">
+      <c r="B109" s="5" t="s">
         <v>221</v>
+      </c>
+      <c r="C109" s="6" t="s">
+        <v>412</v>
+      </c>
+      <c r="D109" s="5" t="s">
+        <v>458</v>
+      </c>
+      <c r="E109" s="6" t="b">
+        <v>1</v>
       </c>
       <c r="F109" t="b">
         <v>0</v>
@@ -3310,6 +3597,9 @@
       <c r="B110" s="3" t="s">
         <v>223</v>
       </c>
+      <c r="C110" t="s">
+        <v>412</v>
+      </c>
       <c r="F110" t="b">
         <v>0</v>
       </c>
@@ -3321,6 +3611,9 @@
       <c r="B111" s="3" t="s">
         <v>225</v>
       </c>
+      <c r="C111" t="s">
+        <v>408</v>
+      </c>
       <c r="F111" t="b">
         <v>1</v>
       </c>
@@ -3332,6 +3625,9 @@
       <c r="B112" s="3" t="s">
         <v>227</v>
       </c>
+      <c r="C112" t="s">
+        <v>408</v>
+      </c>
       <c r="F112" t="b">
         <v>1</v>
       </c>
@@ -3343,6 +3639,9 @@
       <c r="B113" s="3" t="s">
         <v>229</v>
       </c>
+      <c r="C113" t="s">
+        <v>412</v>
+      </c>
       <c r="F113" t="b">
         <v>0</v>
       </c>
@@ -3351,8 +3650,17 @@
       <c r="A114" t="s">
         <v>230</v>
       </c>
-      <c r="B114" s="3" t="s">
+      <c r="B114" s="5" t="s">
         <v>231</v>
+      </c>
+      <c r="C114" s="6" t="s">
+        <v>410</v>
+      </c>
+      <c r="D114" s="5" t="s">
+        <v>459</v>
+      </c>
+      <c r="E114" s="6" t="b">
+        <v>1</v>
       </c>
       <c r="F114" t="b">
         <v>0</v>
@@ -3365,6 +3673,9 @@
       <c r="B115" s="3" t="s">
         <v>233</v>
       </c>
+      <c r="C115" t="s">
+        <v>408</v>
+      </c>
       <c r="F115" t="b">
         <v>1</v>
       </c>
@@ -3376,6 +3687,9 @@
       <c r="B116" s="3" t="s">
         <v>235</v>
       </c>
+      <c r="C116" t="s">
+        <v>412</v>
+      </c>
       <c r="F116" t="b">
         <v>0</v>
       </c>
@@ -3387,6 +3701,12 @@
       <c r="B117" s="3" t="s">
         <v>237</v>
       </c>
+      <c r="C117" t="s">
+        <v>412</v>
+      </c>
+      <c r="D117" s="3" t="s">
+        <v>460</v>
+      </c>
       <c r="F117" t="b">
         <v>0</v>
       </c>
@@ -3398,6 +3718,9 @@
       <c r="B118" s="3" t="s">
         <v>239</v>
       </c>
+      <c r="C118" t="s">
+        <v>408</v>
+      </c>
       <c r="F118" t="b">
         <v>1</v>
       </c>
@@ -3409,6 +3732,9 @@
       <c r="B119" s="3" t="s">
         <v>241</v>
       </c>
+      <c r="C119" t="s">
+        <v>407</v>
+      </c>
       <c r="F119" t="b">
         <v>0</v>
       </c>
@@ -3420,6 +3746,9 @@
       <c r="B120" s="3" t="s">
         <v>243</v>
       </c>
+      <c r="C120" t="s">
+        <v>408</v>
+      </c>
       <c r="F120" t="b">
         <v>1</v>
       </c>
@@ -3431,6 +3760,9 @@
       <c r="B121" s="3" t="s">
         <v>245</v>
       </c>
+      <c r="C121" t="s">
+        <v>408</v>
+      </c>
       <c r="F121" t="b">
         <v>1</v>
       </c>
@@ -3442,6 +3774,9 @@
       <c r="B122" s="3" t="s">
         <v>247</v>
       </c>
+      <c r="C122" t="s">
+        <v>408</v>
+      </c>
       <c r="F122" t="b">
         <v>1</v>
       </c>
@@ -3450,8 +3785,17 @@
       <c r="A123" t="s">
         <v>248</v>
       </c>
-      <c r="B123" s="3" t="s">
+      <c r="B123" s="5" t="s">
         <v>249</v>
+      </c>
+      <c r="C123" s="6" t="s">
+        <v>410</v>
+      </c>
+      <c r="D123" s="5" t="s">
+        <v>461</v>
+      </c>
+      <c r="E123" s="6" t="b">
+        <v>1</v>
       </c>
       <c r="F123" t="b">
         <v>0</v>
@@ -3464,6 +3808,9 @@
       <c r="B124" s="3" t="s">
         <v>251</v>
       </c>
+      <c r="C124" t="s">
+        <v>408</v>
+      </c>
       <c r="F124" t="b">
         <v>1</v>
       </c>
@@ -3472,8 +3819,17 @@
       <c r="A125" t="s">
         <v>252</v>
       </c>
-      <c r="B125" s="3" t="s">
+      <c r="B125" s="5" t="s">
         <v>253</v>
+      </c>
+      <c r="C125" s="6" t="s">
+        <v>410</v>
+      </c>
+      <c r="D125" s="5" t="s">
+        <v>462</v>
+      </c>
+      <c r="E125" s="6" t="b">
+        <v>1</v>
       </c>
       <c r="F125" t="b">
         <v>0</v>
@@ -3486,6 +3842,9 @@
       <c r="B126" s="3" t="s">
         <v>255</v>
       </c>
+      <c r="C126" t="s">
+        <v>408</v>
+      </c>
       <c r="F126" t="b">
         <v>1</v>
       </c>
@@ -3494,8 +3853,17 @@
       <c r="A127" t="s">
         <v>256</v>
       </c>
-      <c r="B127" s="3" t="s">
+      <c r="B127" s="5" t="s">
         <v>257</v>
+      </c>
+      <c r="C127" s="6" t="s">
+        <v>409</v>
+      </c>
+      <c r="D127" s="5" t="s">
+        <v>463</v>
+      </c>
+      <c r="E127" s="6" t="b">
+        <v>1</v>
       </c>
       <c r="F127" t="b">
         <v>1</v>
@@ -3508,6 +3876,9 @@
       <c r="B128" s="3" t="s">
         <v>259</v>
       </c>
+      <c r="C128" t="s">
+        <v>408</v>
+      </c>
       <c r="F128" t="b">
         <v>1</v>
       </c>
@@ -3519,6 +3890,9 @@
       <c r="B129" s="3" t="s">
         <v>261</v>
       </c>
+      <c r="C129" t="s">
+        <v>408</v>
+      </c>
       <c r="F129" t="b">
         <v>1</v>
       </c>
@@ -3530,6 +3904,9 @@
       <c r="B130" s="3" t="s">
         <v>263</v>
       </c>
+      <c r="C130" t="s">
+        <v>408</v>
+      </c>
       <c r="F130" t="b">
         <v>1</v>
       </c>
@@ -3541,6 +3918,9 @@
       <c r="B131" s="3" t="s">
         <v>265</v>
       </c>
+      <c r="C131" t="s">
+        <v>408</v>
+      </c>
       <c r="F131" t="b">
         <v>1</v>
       </c>
@@ -3552,6 +3932,9 @@
       <c r="B132" s="3" t="s">
         <v>267</v>
       </c>
+      <c r="C132" t="s">
+        <v>408</v>
+      </c>
       <c r="F132" t="b">
         <v>1</v>
       </c>
@@ -3563,6 +3946,9 @@
       <c r="B133" s="3" t="s">
         <v>269</v>
       </c>
+      <c r="C133" t="s">
+        <v>408</v>
+      </c>
       <c r="F133" t="b">
         <v>1</v>
       </c>
@@ -3574,6 +3960,9 @@
       <c r="B134" s="3" t="s">
         <v>271</v>
       </c>
+      <c r="C134" t="s">
+        <v>408</v>
+      </c>
       <c r="F134" t="b">
         <v>1</v>
       </c>
@@ -3585,6 +3974,9 @@
       <c r="B135" s="3" t="s">
         <v>273</v>
       </c>
+      <c r="C135" t="s">
+        <v>408</v>
+      </c>
       <c r="F135" t="b">
         <v>1</v>
       </c>
@@ -3596,6 +3988,9 @@
       <c r="B136" s="3" t="s">
         <v>275</v>
       </c>
+      <c r="C136" t="s">
+        <v>408</v>
+      </c>
       <c r="F136" t="b">
         <v>1</v>
       </c>
@@ -3607,6 +4002,9 @@
       <c r="B137" s="3" t="s">
         <v>277</v>
       </c>
+      <c r="C137" t="s">
+        <v>408</v>
+      </c>
       <c r="F137" t="b">
         <v>1</v>
       </c>
@@ -3618,6 +4016,9 @@
       <c r="B138" s="3" t="s">
         <v>279</v>
       </c>
+      <c r="C138" t="s">
+        <v>408</v>
+      </c>
       <c r="F138" t="b">
         <v>1</v>
       </c>
@@ -3629,6 +4030,9 @@
       <c r="B139" s="3" t="s">
         <v>281</v>
       </c>
+      <c r="C139" t="s">
+        <v>412</v>
+      </c>
       <c r="F139" t="b">
         <v>0</v>
       </c>
@@ -3640,6 +4044,9 @@
       <c r="B140" s="3" t="s">
         <v>283</v>
       </c>
+      <c r="C140" t="s">
+        <v>408</v>
+      </c>
       <c r="F140" t="b">
         <v>1</v>
       </c>
@@ -3651,6 +4058,9 @@
       <c r="B141" s="3" t="s">
         <v>285</v>
       </c>
+      <c r="C141" t="s">
+        <v>408</v>
+      </c>
       <c r="F141" t="b">
         <v>1</v>
       </c>
@@ -3662,6 +4072,9 @@
       <c r="B142" s="3" t="s">
         <v>287</v>
       </c>
+      <c r="C142" t="s">
+        <v>408</v>
+      </c>
       <c r="F142" t="b">
         <v>1</v>
       </c>
@@ -3673,6 +4086,9 @@
       <c r="B143" s="3" t="s">
         <v>289</v>
       </c>
+      <c r="C143" t="s">
+        <v>408</v>
+      </c>
       <c r="F143" t="b">
         <v>1</v>
       </c>
@@ -3684,6 +4100,9 @@
       <c r="B144" s="3" t="s">
         <v>291</v>
       </c>
+      <c r="C144" t="s">
+        <v>408</v>
+      </c>
       <c r="F144" t="b">
         <v>1</v>
       </c>
@@ -3695,6 +4114,9 @@
       <c r="B145" s="3" t="s">
         <v>293</v>
       </c>
+      <c r="C145" t="s">
+        <v>412</v>
+      </c>
       <c r="F145" t="b">
         <v>0</v>
       </c>
@@ -3706,16 +4128,28 @@
       <c r="B146" s="3" t="s">
         <v>295</v>
       </c>
+      <c r="C146" t="s">
+        <v>408</v>
+      </c>
       <c r="F146" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="147" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:6" ht="48" x14ac:dyDescent="0.2">
       <c r="A147" t="s">
         <v>296</v>
       </c>
-      <c r="B147" s="3" t="s">
+      <c r="B147" s="5" t="s">
         <v>297</v>
+      </c>
+      <c r="C147" s="6" t="s">
+        <v>409</v>
+      </c>
+      <c r="D147" s="5" t="s">
+        <v>464</v>
+      </c>
+      <c r="E147" s="6" t="b">
+        <v>1</v>
       </c>
       <c r="F147" t="b">
         <v>1</v>
@@ -3728,6 +4162,12 @@
       <c r="B148" s="3" t="s">
         <v>299</v>
       </c>
+      <c r="C148" t="s">
+        <v>412</v>
+      </c>
+      <c r="D148" s="3" t="s">
+        <v>465</v>
+      </c>
       <c r="F148" t="b">
         <v>1</v>
       </c>
@@ -3739,6 +4179,9 @@
       <c r="B149" s="3" t="s">
         <v>301</v>
       </c>
+      <c r="C149" t="s">
+        <v>408</v>
+      </c>
       <c r="F149" t="b">
         <v>1</v>
       </c>
@@ -3750,6 +4193,9 @@
       <c r="B150" s="3" t="s">
         <v>303</v>
       </c>
+      <c r="C150" t="s">
+        <v>408</v>
+      </c>
       <c r="F150" t="b">
         <v>1</v>
       </c>
@@ -3758,8 +4204,15 @@
       <c r="A151" t="s">
         <v>304</v>
       </c>
-      <c r="B151" s="3" t="s">
+      <c r="B151" s="5" t="s">
         <v>305</v>
+      </c>
+      <c r="C151" s="6" t="s">
+        <v>408</v>
+      </c>
+      <c r="D151" s="5"/>
+      <c r="E151" s="6" t="b">
+        <v>1</v>
       </c>
       <c r="F151" t="b">
         <v>1</v>
@@ -3772,6 +4225,9 @@
       <c r="B152" s="3" t="s">
         <v>307</v>
       </c>
+      <c r="C152" t="s">
+        <v>412</v>
+      </c>
       <c r="F152" t="b">
         <v>0</v>
       </c>
@@ -3780,8 +4236,13 @@
       <c r="A153" t="s">
         <v>308</v>
       </c>
-      <c r="B153" s="3" t="s">
+      <c r="B153" s="5" t="s">
         <v>309</v>
+      </c>
+      <c r="C153" s="6"/>
+      <c r="D153" s="5"/>
+      <c r="E153" s="6" t="b">
+        <v>1</v>
       </c>
       <c r="F153" t="b">
         <v>0</v>
@@ -3794,6 +4255,9 @@
       <c r="B154" s="3" t="s">
         <v>311</v>
       </c>
+      <c r="C154" t="s">
+        <v>412</v>
+      </c>
       <c r="F154" t="b">
         <v>0</v>
       </c>
@@ -3805,6 +4269,9 @@
       <c r="B155" s="3" t="s">
         <v>313</v>
       </c>
+      <c r="C155" t="s">
+        <v>408</v>
+      </c>
       <c r="F155" t="b">
         <v>1</v>
       </c>
@@ -4317,7 +4784,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C1:C1048576" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C1:C83 C85:C145 C147:C1048576" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>$G$2:$G$7</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Add Main4 analysis and update Main analysis
</commit_message>
<xml_diff>
--- a/Annotation_Main/Main4/Main4_Katja.xlsx
+++ b/Annotation_Main/Main4/Main4_Katja.xlsx
@@ -1,26 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="11012"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/katja/Dropbox/Doktorat/ParlaMint/Sentiment_annotation-speeches/Annotation_Main/Main4/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\katjam\Dropbox\Doktorat\ParlaMint\Sentiment_annotation-speeches\Annotation_Main\Main4\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEBCA7C7-0E5F-AF4D-AEE2-45B9BD62C7DC}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="16220" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="495" windowWidth="28800" windowHeight="16215"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="152511"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="618" uniqueCount="466">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="682" uniqueCount="482">
   <si>
     <t>ID</t>
   </si>
@@ -1270,12 +1269,6 @@
     <t xml:space="preserve">At the end there is a slight negative connotation, but the overall tone of the speech is positive, albeit a bit weak. </t>
   </si>
   <si>
-    <t>The speaker details problems and possible solutions on the systemic corruption. The topic is obviously negative, but it is hard to detect the sentiment in the speech itself, as it seems relatively negative (though a bit weak), and at the same time, a bit neutral (speaker offers no position, no explicit proposal, just "what can be done").   It could be just directly Negative (but again, a bit weak).</t>
-  </si>
-  <si>
-    <t>Uf, the speech is defensive and at beginning and end accompanied with pretty harsh (and sarcastic) words. The middle is detailing facts (as per the speaker) and is relatively neutral. However, to me, the overall speech still seems very negative, but could maybe also be M_Negative.</t>
-  </si>
-  <si>
     <t>Speaker presenting and explaining the bill. I do not sense explicit speaker position or sentiment, mostly as we cannot discern from the text, if the speaker belongs to the Government or not. So due to the above, I would say this is relatively neutral.</t>
   </si>
   <si>
@@ -1354,9 +1347,6 @@
     <t xml:space="preserve">To me this feels slightly defensive, and while there are some positive points in the speech. </t>
   </si>
   <si>
-    <t>Just a statement but with slight negative connotation.</t>
-  </si>
-  <si>
     <t>Could also be Negative.</t>
   </si>
   <si>
@@ -1411,19 +1401,76 @@
     <t xml:space="preserve">Majority of speech positive, but in the second part the sentiment turns to negative (..."Kljub temu pa smo v  poslanski skupini ugotovili vrsto pomanjkljivosti). </t>
   </si>
   <si>
-    <t>Could also be P_Neutral</t>
-  </si>
-  <si>
     <t>Seems like a warning to the speaker. Could just as well be directly Negative.</t>
   </si>
   <si>
-    <t>Uffff, negative (probably procedural).</t>
+    <t>Seems aggressive and accusatory.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The sentiment shifts at several points in the speech. </t>
+  </si>
+  <si>
+    <t>The two last sentences are a bit more positive in tone, as the speaker calls for support in the name of his PS. But overall the speech is negative. Could also be M_Negative.</t>
+  </si>
+  <si>
+    <t>Negative (though probably procedural).</t>
+  </si>
+  <si>
+    <t>Seems forceful</t>
+  </si>
+  <si>
+    <t>Defensive and negative</t>
+  </si>
+  <si>
+    <t>First part positive and second negative.</t>
+  </si>
+  <si>
+    <t>At the end there is a positive sentence, but with call for support of her proposal, but the entire speech is negative.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">While generally positive speech in support of (their own amandma), but the speaker still adds negative insertions, relating to the opposition and their previous proposal. </t>
+  </si>
+  <si>
+    <t>Either neutral or mixed, not sure</t>
+  </si>
+  <si>
+    <t>Either Negative or N_Neutral. Could be just an explanation or a defensive stance.</t>
+  </si>
+  <si>
+    <t>Interpelation - very negative, and even though the speech contains also features of some positive changes they have made, this is done in defence.</t>
+  </si>
+  <si>
+    <t>Statement, but with a negative connotation</t>
+  </si>
+  <si>
+    <t>Not sure if full weak positive or mixed positive</t>
+  </si>
+  <si>
+    <t>Either N_Neutral or Negative</t>
+  </si>
+  <si>
+    <t>Weak negative, but still negative. Speaker outlines all of the empty promises that were given and are still not fulfilled.</t>
+  </si>
+  <si>
+    <t>The speaker details problems and possible solutions on the systemic corruption. The topic is obviously negative, but the speech itself just outlines the points that we already have in place and in the second part starts pointing out different points that still need to be addressed. So while this seems weakly positive or even neutral, it still has some negative connotation in it. The speaker does not offer explicit positions and just talks about "what needs to be done". I have a really hard time interpreting the sentiment in this speech.</t>
+  </si>
+  <si>
+    <t>The speech is defensive and at beginning and end accompanied with pretty harsh (and sarcastic) words. The middle is detailing facts (as per the speaker) and is relatively neutral.</t>
+  </si>
+  <si>
+    <t>Negative topic, and the speech itself is not exactly positive. The speaker is aware of the problematic aspects and hopes for better future. Could also be Negative.</t>
+  </si>
+  <si>
+    <t>Could also be N_Neutral, no context.</t>
+  </si>
+  <si>
+    <t>The speech seems a bit defensive and negative.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -1439,18 +1486,12 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -1515,13 +1556,13 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Navadno" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -1820,19 +1861,19 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G201"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:H201"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="39.1640625" hidden="1" customWidth="1"/>
-    <col min="2" max="2" width="124.6640625" style="3" customWidth="1"/>
+    <col min="1" max="1" width="39.140625" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="124.7109375" style="3" customWidth="1"/>
     <col min="3" max="3" width="27" customWidth="1"/>
-    <col min="4" max="4" width="22.83203125" style="3" customWidth="1"/>
-    <col min="6" max="6" width="0" hidden="1" customWidth="1"/>
-    <col min="7" max="7" width="18.5" hidden="1" customWidth="1"/>
+    <col min="4" max="4" width="22.85546875" style="3" customWidth="1"/>
+    <col min="6" max="6" width="6.140625" hidden="1" customWidth="1"/>
+    <col min="7" max="7" width="18.42578125" hidden="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1855,7 +1896,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>6</v>
       </c>
@@ -1872,7 +1913,7 @@
         <v>407</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="192" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:7" ht="210" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>8</v>
       </c>
@@ -1895,7 +1936,7 @@
         <v>408</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>10</v>
       </c>
@@ -1912,7 +1953,7 @@
         <v>409</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="160" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" ht="180" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>12</v>
       </c>
@@ -1932,7 +1973,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="335" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" ht="375" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>14</v>
       </c>
@@ -1952,7 +1993,7 @@
         <v>411</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="240" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" ht="270" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>16</v>
       </c>
@@ -1969,7 +2010,7 @@
         <v>412</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="335" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" ht="375" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>18</v>
       </c>
@@ -1983,27 +2024,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="380" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>20</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="C9" s="8" t="s">
         <v>411</v>
       </c>
-      <c r="D9" s="5" t="s">
-        <v>416</v>
-      </c>
-      <c r="E9" s="6" t="b">
+      <c r="D9" s="7" t="s">
+        <v>477</v>
+      </c>
+      <c r="E9" s="8" t="b">
         <v>1</v>
       </c>
       <c r="F9" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" ht="30" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>22</v>
       </c>
@@ -2017,47 +2058,45 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="176" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" ht="180" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>24</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="C11" s="6" t="s">
-        <v>412</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>417</v>
-      </c>
-      <c r="E11" s="6" t="b">
-        <v>1</v>
-      </c>
+      <c r="C11" s="8" t="s">
+        <v>412</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>478</v>
+      </c>
+      <c r="E11" s="8"/>
       <c r="F11" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="176" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" ht="195" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>26</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="C12" s="6" t="s">
-        <v>408</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>418</v>
-      </c>
-      <c r="E12" s="6" t="b">
+      <c r="C12" s="8" t="s">
+        <v>408</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>416</v>
+      </c>
+      <c r="E12" s="8" t="b">
         <v>1</v>
       </c>
       <c r="F12" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="380" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>28</v>
       </c>
@@ -2068,13 +2107,13 @@
         <v>412</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>419</v>
+        <v>417</v>
       </c>
       <c r="F13" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="16" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>30</v>
       </c>
@@ -2088,7 +2127,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="128" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" ht="150" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>32</v>
       </c>
@@ -2102,7 +2141,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="365" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>34</v>
       </c>
@@ -2113,13 +2152,13 @@
         <v>410</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>420</v>
+        <v>418</v>
       </c>
       <c r="F16" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>36</v>
       </c>
@@ -2130,7 +2169,7 @@
         <v>412</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>421</v>
+        <v>419</v>
       </c>
       <c r="E17" t="b">
         <v>1</v>
@@ -2139,27 +2178,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="80" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6" ht="90" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>38</v>
       </c>
-      <c r="B18" s="5" t="s">
+      <c r="B18" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="C18" s="6" t="s">
-        <v>409</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>422</v>
-      </c>
-      <c r="E18" s="6" t="b">
+      <c r="C18" s="8" t="s">
+        <v>412</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>420</v>
+      </c>
+      <c r="E18" s="8" t="b">
         <v>1</v>
       </c>
       <c r="F18" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="160" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6" ht="180" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>40</v>
       </c>
@@ -2170,13 +2209,13 @@
         <v>412</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>423</v>
+        <v>421</v>
       </c>
       <c r="F19" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="80" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6" ht="90" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>42</v>
       </c>
@@ -2190,27 +2229,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="350" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6" ht="405" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>44</v>
       </c>
-      <c r="B21" s="5" t="s">
+      <c r="B21" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="C21" s="6" t="s">
-        <v>412</v>
-      </c>
-      <c r="D21" s="5" t="s">
-        <v>424</v>
-      </c>
-      <c r="E21" s="6" t="b">
+      <c r="C21" s="8" t="s">
+        <v>412</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>422</v>
+      </c>
+      <c r="E21" s="8" t="b">
         <v>1</v>
       </c>
       <c r="F21" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="112" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6" ht="120" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>46</v>
       </c>
@@ -2224,27 +2263,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="350" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:6" ht="390" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>48</v>
       </c>
-      <c r="B23" s="5" t="s">
+      <c r="B23" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="C23" s="6" t="s">
+      <c r="C23" s="8" t="s">
         <v>411</v>
       </c>
-      <c r="D23" s="5" t="s">
-        <v>425</v>
-      </c>
-      <c r="E23" s="6" t="b">
+      <c r="D23" s="7" t="s">
+        <v>423</v>
+      </c>
+      <c r="E23" s="8" t="b">
         <v>1</v>
       </c>
       <c r="F23" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:6" ht="240" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:6" ht="270" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>50</v>
       </c>
@@ -2255,13 +2294,13 @@
         <v>410</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>427</v>
+        <v>425</v>
       </c>
       <c r="F24" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:6" ht="48" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>52</v>
       </c>
@@ -2272,7 +2311,7 @@
         <v>409</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>426</v>
+        <v>424</v>
       </c>
       <c r="E25" t="b">
         <v>1</v>
@@ -2281,23 +2320,25 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:6" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>54</v>
       </c>
-      <c r="B26" s="7" t="s">
+      <c r="B26" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="C26" s="8"/>
-      <c r="D26" s="7" t="s">
-        <v>428</v>
-      </c>
-      <c r="E26" s="8"/>
+      <c r="C26" s="6" t="s">
+        <v>408</v>
+      </c>
+      <c r="D26" s="5" t="s">
+        <v>426</v>
+      </c>
+      <c r="E26" s="6"/>
       <c r="F26" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>56</v>
       </c>
@@ -2311,7 +2352,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>58</v>
       </c>
@@ -2325,27 +2366,27 @@
         <v>1</v>
       </c>
     </row>
-    <row r="29" spans="1:6" ht="240" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:6" ht="270" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>60</v>
       </c>
-      <c r="B29" s="5" t="s">
+      <c r="B29" s="7" t="s">
         <v>61</v>
       </c>
-      <c r="C29" s="6" t="s">
+      <c r="C29" s="8" t="s">
         <v>411</v>
       </c>
-      <c r="D29" s="5" t="s">
-        <v>429</v>
-      </c>
-      <c r="E29" s="6" t="b">
+      <c r="D29" s="7" t="s">
+        <v>427</v>
+      </c>
+      <c r="E29" s="8" t="b">
         <v>1</v>
       </c>
       <c r="F29" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>62</v>
       </c>
@@ -2359,7 +2400,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:6" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>64</v>
       </c>
@@ -2370,24 +2411,24 @@
         <v>411</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>430</v>
+        <v>428</v>
       </c>
       <c r="F31" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:6" ht="64" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:6" ht="75" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>66</v>
       </c>
-      <c r="B32" s="5" t="s">
+      <c r="B32" s="7" t="s">
         <v>67</v>
       </c>
-      <c r="C32" s="6" t="s">
-        <v>408</v>
-      </c>
-      <c r="D32" s="5" t="s">
-        <v>431</v>
+      <c r="C32" s="8" t="s">
+        <v>408</v>
+      </c>
+      <c r="D32" s="7" t="s">
+        <v>429</v>
       </c>
       <c r="E32" t="b">
         <v>1</v>
@@ -2396,7 +2437,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:6" ht="256" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:6" ht="285" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>68</v>
       </c>
@@ -2410,7 +2451,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>70</v>
       </c>
@@ -2424,7 +2465,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="35" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>72</v>
       </c>
@@ -2438,7 +2479,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:6" ht="96" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:6" ht="105" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>74</v>
       </c>
@@ -2452,7 +2493,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>76</v>
       </c>
@@ -2466,7 +2507,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>78</v>
       </c>
@@ -2480,7 +2521,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:6" ht="176" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:6" ht="195" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>80</v>
       </c>
@@ -2491,13 +2532,13 @@
         <v>412</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>432</v>
+        <v>430</v>
       </c>
       <c r="F39" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:6" ht="48" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>82</v>
       </c>
@@ -2508,13 +2549,13 @@
         <v>412</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>433</v>
+        <v>431</v>
       </c>
       <c r="F40" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>84</v>
       </c>
@@ -2528,7 +2569,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:6" ht="64" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>86</v>
       </c>
@@ -2539,13 +2580,13 @@
         <v>409</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>434</v>
+        <v>432</v>
       </c>
       <c r="F42" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>88</v>
       </c>
@@ -2559,27 +2600,27 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:6" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>90</v>
       </c>
-      <c r="B44" s="5" t="s">
+      <c r="B44" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="C44" s="6" t="s">
+      <c r="C44" s="8" t="s">
         <v>411</v>
       </c>
-      <c r="D44" s="5" t="s">
-        <v>435</v>
-      </c>
-      <c r="E44" s="6" t="b">
+      <c r="D44" s="7" t="s">
+        <v>433</v>
+      </c>
+      <c r="E44" s="8" t="b">
         <v>1</v>
       </c>
       <c r="F44" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>92</v>
       </c>
@@ -2593,7 +2634,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>94</v>
       </c>
@@ -2607,7 +2648,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="47" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>96</v>
       </c>
@@ -2621,7 +2662,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:6" ht="48" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>98</v>
       </c>
@@ -2635,7 +2676,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="1:6" ht="48" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>100</v>
       </c>
@@ -2649,7 +2690,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="50" spans="1:6" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>102</v>
       </c>
@@ -2663,7 +2704,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:6" ht="208" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:6" ht="225" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>104</v>
       </c>
@@ -2674,7 +2715,7 @@
         <v>412</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>436</v>
+        <v>434</v>
       </c>
       <c r="E51" t="b">
         <v>1</v>
@@ -2683,7 +2724,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:6" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>106</v>
       </c>
@@ -2694,13 +2735,13 @@
         <v>412</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>437</v>
+        <v>435</v>
       </c>
       <c r="F52" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>108</v>
       </c>
@@ -2714,7 +2755,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="54" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A54" t="s">
         <v>110</v>
       </c>
@@ -2728,7 +2769,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A55" t="s">
         <v>112</v>
       </c>
@@ -2742,7 +2783,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="56" spans="1:6" ht="128" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:6" ht="135" x14ac:dyDescent="0.25">
       <c r="A56" t="s">
         <v>114</v>
       </c>
@@ -2753,13 +2794,13 @@
         <v>410</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>438</v>
+        <v>436</v>
       </c>
       <c r="F56" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:6" ht="48" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A57" t="s">
         <v>116</v>
       </c>
@@ -2770,13 +2811,13 @@
         <v>412</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>439</v>
+        <v>437</v>
       </c>
       <c r="F57" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A58" t="s">
         <v>118</v>
       </c>
@@ -2790,7 +2831,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="59" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A59" t="s">
         <v>120</v>
       </c>
@@ -2804,7 +2845,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="60" spans="1:6" ht="48" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A60" t="s">
         <v>122</v>
       </c>
@@ -2818,7 +2859,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="61" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A61" t="s">
         <v>124</v>
       </c>
@@ -2832,7 +2873,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="62" spans="1:6" ht="64" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:6" ht="75" x14ac:dyDescent="0.25">
       <c r="A62" t="s">
         <v>126</v>
       </c>
@@ -2843,7 +2884,7 @@
         <v>408</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>440</v>
+        <v>438</v>
       </c>
       <c r="E62" t="b">
         <v>1</v>
@@ -2852,7 +2893,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="63" spans="1:6" ht="192" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:6" ht="225" x14ac:dyDescent="0.25">
       <c r="A63" t="s">
         <v>128</v>
       </c>
@@ -2863,13 +2904,13 @@
         <v>412</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>441</v>
+        <v>439</v>
       </c>
       <c r="F63" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:6" ht="335" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:6" ht="360" x14ac:dyDescent="0.25">
       <c r="A64" t="s">
         <v>130</v>
       </c>
@@ -2880,7 +2921,7 @@
         <v>411</v>
       </c>
       <c r="D64" s="3" t="s">
-        <v>442</v>
+        <v>440</v>
       </c>
       <c r="E64" t="b">
         <v>1</v>
@@ -2889,7 +2930,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:6" ht="176" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:8" ht="195" x14ac:dyDescent="0.25">
       <c r="A65" t="s">
         <v>132</v>
       </c>
@@ -2900,13 +2941,13 @@
         <v>411</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>443</v>
+        <v>441</v>
       </c>
       <c r="F65" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66" t="s">
         <v>134</v>
       </c>
@@ -2920,24 +2961,27 @@
         <v>1</v>
       </c>
     </row>
-    <row r="67" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67" t="s">
         <v>136</v>
       </c>
-      <c r="B67" s="5" t="s">
+      <c r="B67" s="7" t="s">
         <v>137</v>
       </c>
-      <c r="C67" s="6" t="s">
-        <v>409</v>
-      </c>
-      <c r="D67" s="5" t="s">
-        <v>444</v>
+      <c r="C67" s="8" t="s">
+        <v>412</v>
+      </c>
+      <c r="D67" s="7" t="s">
+        <v>465</v>
+      </c>
+      <c r="E67" s="8" t="b">
+        <v>1</v>
       </c>
       <c r="F67" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68" t="s">
         <v>138</v>
       </c>
@@ -2951,7 +2995,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A69" t="s">
         <v>140</v>
       </c>
@@ -2965,7 +3009,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="70" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70" t="s">
         <v>142</v>
       </c>
@@ -2976,7 +3020,7 @@
         <v>409</v>
       </c>
       <c r="D70" s="3" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
       <c r="E70" t="b">
         <v>1</v>
@@ -2985,23 +3029,23 @@
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71" t="s">
         <v>144</v>
       </c>
-      <c r="B71" s="5" t="s">
+      <c r="B71" s="7" t="s">
         <v>145</v>
       </c>
-      <c r="C71" s="6" t="s">
-        <v>412</v>
-      </c>
-      <c r="D71" s="5"/>
-      <c r="E71" s="6"/>
+      <c r="C71" s="8" t="s">
+        <v>412</v>
+      </c>
+      <c r="D71" s="7"/>
+      <c r="E71" s="8"/>
       <c r="F71" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="72" spans="1:6" ht="112" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:8" ht="120" x14ac:dyDescent="0.25">
       <c r="A72" t="s">
         <v>146</v>
       </c>
@@ -3012,13 +3056,13 @@
         <v>407</v>
       </c>
       <c r="D72" s="3" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
       <c r="F72" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="1:6" ht="176" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:8" ht="195" x14ac:dyDescent="0.25">
       <c r="A73" t="s">
         <v>148</v>
       </c>
@@ -3029,13 +3073,13 @@
         <v>411</v>
       </c>
       <c r="D73" s="3" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
       <c r="F73" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="74" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74" t="s">
         <v>150</v>
       </c>
@@ -3049,7 +3093,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="75" spans="1:6" ht="144" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:8" ht="165" x14ac:dyDescent="0.25">
       <c r="A75" t="s">
         <v>152</v>
       </c>
@@ -3060,13 +3104,13 @@
         <v>407</v>
       </c>
       <c r="D75" s="3" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
       <c r="F75" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="76" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A76" t="s">
         <v>154</v>
       </c>
@@ -3080,37 +3124,39 @@
         <v>1</v>
       </c>
     </row>
-    <row r="77" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A77" t="s">
         <v>156</v>
       </c>
-      <c r="B77" s="5" t="s">
+      <c r="B77" s="7" t="s">
         <v>157</v>
       </c>
-      <c r="C77" s="6" t="s">
+      <c r="C77" s="8" t="s">
         <v>409</v>
       </c>
-      <c r="D77" s="5"/>
+      <c r="D77" s="7"/>
+      <c r="E77" s="8"/>
       <c r="F77" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="78" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A78" t="s">
         <v>158</v>
       </c>
-      <c r="B78" s="5" t="s">
+      <c r="B78" s="7" t="s">
         <v>159</v>
       </c>
-      <c r="C78" s="6" t="s">
-        <v>408</v>
-      </c>
-      <c r="D78" s="5"/>
+      <c r="C78" s="8" t="s">
+        <v>408</v>
+      </c>
+      <c r="D78" s="7"/>
+      <c r="E78" s="8"/>
       <c r="F78" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="79" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A79" t="s">
         <v>160</v>
       </c>
@@ -3124,27 +3170,29 @@
         <v>1</v>
       </c>
     </row>
-    <row r="80" spans="1:6" ht="80" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="A80" t="s">
         <v>162</v>
       </c>
-      <c r="B80" s="5" t="s">
+      <c r="B80" s="7" t="s">
         <v>163</v>
       </c>
-      <c r="C80" s="6" t="s">
-        <v>412</v>
-      </c>
-      <c r="D80" s="5" t="s">
-        <v>449</v>
-      </c>
-      <c r="E80" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="F80" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="81" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="C80" s="8" t="s">
+        <v>412</v>
+      </c>
+      <c r="D80" s="7" t="s">
+        <v>446</v>
+      </c>
+      <c r="E80" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="F80" s="8" t="b">
+        <v>0</v>
+      </c>
+      <c r="G80" s="8"/>
+      <c r="H80" s="8"/>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
         <v>164</v>
       </c>
@@ -3158,7 +3206,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="82" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A82" t="s">
         <v>166</v>
       </c>
@@ -3172,7 +3220,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="83" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A83" t="s">
         <v>168</v>
       </c>
@@ -3186,7 +3234,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="84" spans="1:6" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A84" t="s">
         <v>170</v>
       </c>
@@ -3200,7 +3248,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A85" t="s">
         <v>172</v>
       </c>
@@ -3214,7 +3262,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="86" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A86" t="s">
         <v>174</v>
       </c>
@@ -3228,47 +3276,47 @@
         <v>1</v>
       </c>
     </row>
-    <row r="87" spans="1:6" ht="112" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:6" ht="120" x14ac:dyDescent="0.25">
       <c r="A87" t="s">
         <v>176</v>
       </c>
-      <c r="B87" s="5" t="s">
+      <c r="B87" s="7" t="s">
         <v>177</v>
       </c>
-      <c r="C87" s="6" t="s">
+      <c r="C87" s="8" t="s">
         <v>410</v>
       </c>
-      <c r="D87" s="5" t="s">
-        <v>450</v>
-      </c>
-      <c r="E87" s="6" t="b">
+      <c r="D87" s="7" t="s">
+        <v>447</v>
+      </c>
+      <c r="E87" s="8" t="b">
         <v>1</v>
       </c>
       <c r="F87" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:6" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
         <v>178</v>
       </c>
-      <c r="B88" s="5" t="s">
+      <c r="B88" s="7" t="s">
         <v>179</v>
       </c>
-      <c r="C88" s="6" t="s">
+      <c r="C88" s="8" t="s">
         <v>411</v>
       </c>
-      <c r="D88" s="5" t="s">
-        <v>451</v>
-      </c>
-      <c r="E88" s="6" t="b">
+      <c r="D88" s="7" t="s">
+        <v>448</v>
+      </c>
+      <c r="E88" s="8" t="b">
         <v>1</v>
       </c>
       <c r="F88" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="89" spans="1:6" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A89" t="s">
         <v>180</v>
       </c>
@@ -3279,13 +3327,13 @@
         <v>412</v>
       </c>
       <c r="D89" s="3" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
       <c r="F89" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="90" spans="1:6" ht="48" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A90" t="s">
         <v>182</v>
       </c>
@@ -3296,13 +3344,13 @@
         <v>408</v>
       </c>
       <c r="D90" s="3" t="s">
-        <v>453</v>
+        <v>450</v>
       </c>
       <c r="F90" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A91" t="s">
         <v>184</v>
       </c>
@@ -3316,7 +3364,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="92" spans="1:6" ht="380" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A92" t="s">
         <v>186</v>
       </c>
@@ -3330,22 +3378,23 @@
         <v>0</v>
       </c>
     </row>
-    <row r="93" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A93" t="s">
         <v>188</v>
       </c>
-      <c r="B93" s="5" t="s">
+      <c r="B93" s="7" t="s">
         <v>189</v>
       </c>
-      <c r="C93" s="6" t="s">
+      <c r="C93" s="8" t="s">
         <v>409</v>
       </c>
-      <c r="D93" s="5"/>
+      <c r="D93" s="7"/>
+      <c r="E93" s="8"/>
       <c r="F93" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="94" spans="1:6" ht="48" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A94" t="s">
         <v>190</v>
       </c>
@@ -3356,13 +3405,13 @@
         <v>412</v>
       </c>
       <c r="D94" s="3" t="s">
-        <v>456</v>
+        <v>453</v>
       </c>
       <c r="F94" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="95" spans="1:6" ht="128" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:6" ht="150" x14ac:dyDescent="0.25">
       <c r="A95" t="s">
         <v>192</v>
       </c>
@@ -3373,7 +3422,7 @@
         <v>411</v>
       </c>
       <c r="D95" s="3" t="s">
-        <v>454</v>
+        <v>451</v>
       </c>
       <c r="E95" t="b">
         <v>1</v>
@@ -3382,7 +3431,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="96" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A96" t="s">
         <v>194</v>
       </c>
@@ -3396,7 +3445,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="97" spans="1:6" ht="48" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A97" t="s">
         <v>196</v>
       </c>
@@ -3407,13 +3456,13 @@
         <v>412</v>
       </c>
       <c r="D97" s="3" t="s">
-        <v>455</v>
+        <v>452</v>
       </c>
       <c r="F97" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="98" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A98" t="s">
         <v>198</v>
       </c>
@@ -3427,7 +3476,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="99" spans="1:6" ht="64" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:6" ht="75" x14ac:dyDescent="0.25">
       <c r="A99" t="s">
         <v>200</v>
       </c>
@@ -3441,7 +3490,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="100" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A100" t="s">
         <v>202</v>
       </c>
@@ -3455,7 +3504,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="101" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A101" t="s">
         <v>204</v>
       </c>
@@ -3469,7 +3518,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="102" spans="1:6" ht="240" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:6" ht="255" x14ac:dyDescent="0.25">
       <c r="A102" t="s">
         <v>206</v>
       </c>
@@ -3483,7 +3532,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="103" spans="1:6" ht="192" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:6" ht="210" x14ac:dyDescent="0.25">
       <c r="A103" t="s">
         <v>208</v>
       </c>
@@ -3497,7 +3546,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A104" t="s">
         <v>210</v>
       </c>
@@ -3511,7 +3560,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="105" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A105" t="s">
         <v>212</v>
       </c>
@@ -3525,7 +3574,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="106" spans="1:6" ht="48" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A106" t="s">
         <v>214</v>
       </c>
@@ -3539,7 +3588,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A107" t="s">
         <v>216</v>
       </c>
@@ -3553,7 +3602,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="108" spans="1:6" ht="160" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:6" ht="180" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
         <v>218</v>
       </c>
@@ -3564,33 +3613,33 @@
         <v>412</v>
       </c>
       <c r="D108" s="3" t="s">
-        <v>457</v>
+        <v>454</v>
       </c>
       <c r="F108" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="109" spans="1:6" ht="96" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:6" ht="105" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
         <v>220</v>
       </c>
-      <c r="B109" s="5" t="s">
+      <c r="B109" s="7" t="s">
         <v>221</v>
       </c>
-      <c r="C109" s="6" t="s">
-        <v>412</v>
-      </c>
-      <c r="D109" s="5" t="s">
-        <v>458</v>
-      </c>
-      <c r="E109" s="6" t="b">
+      <c r="C109" s="8" t="s">
+        <v>412</v>
+      </c>
+      <c r="D109" s="7" t="s">
+        <v>455</v>
+      </c>
+      <c r="E109" s="8" t="b">
         <v>1</v>
       </c>
       <c r="F109" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:6" ht="304" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:6" ht="345" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
         <v>222</v>
       </c>
@@ -3604,7 +3653,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="111" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
         <v>224</v>
       </c>
@@ -3618,7 +3667,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="112" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
         <v>226</v>
       </c>
@@ -3632,7 +3681,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="113" spans="1:6" ht="192" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:8" ht="210" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
         <v>228</v>
       </c>
@@ -3646,27 +3695,29 @@
         <v>0</v>
       </c>
     </row>
-    <row r="114" spans="1:6" ht="80" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
         <v>230</v>
       </c>
-      <c r="B114" s="5" t="s">
+      <c r="B114" s="7" t="s">
         <v>231</v>
       </c>
-      <c r="C114" s="6" t="s">
+      <c r="C114" s="8" t="s">
         <v>410</v>
       </c>
-      <c r="D114" s="5" t="s">
-        <v>459</v>
-      </c>
-      <c r="E114" s="6" t="b">
-        <v>1</v>
-      </c>
-      <c r="F114" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="115" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+      <c r="D114" s="7" t="s">
+        <v>456</v>
+      </c>
+      <c r="E114" s="8" t="b">
+        <v>1</v>
+      </c>
+      <c r="F114" s="8" t="b">
+        <v>0</v>
+      </c>
+      <c r="G114" s="8"/>
+      <c r="H114" s="8"/>
+    </row>
+    <row r="115" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A115" t="s">
         <v>232</v>
       </c>
@@ -3680,7 +3731,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="116" spans="1:6" ht="128" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:8" ht="150" x14ac:dyDescent="0.25">
       <c r="A116" t="s">
         <v>234</v>
       </c>
@@ -3694,7 +3745,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="117" spans="1:6" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:8" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A117" t="s">
         <v>236</v>
       </c>
@@ -3705,13 +3756,13 @@
         <v>412</v>
       </c>
       <c r="D117" s="3" t="s">
-        <v>460</v>
+        <v>457</v>
       </c>
       <c r="F117" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="118" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A118" t="s">
         <v>238</v>
       </c>
@@ -3725,7 +3776,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="119" spans="1:6" ht="112" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:8" ht="120" x14ac:dyDescent="0.25">
       <c r="A119" t="s">
         <v>240</v>
       </c>
@@ -3739,7 +3790,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="120" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A120" t="s">
         <v>242</v>
       </c>
@@ -3753,7 +3804,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="121" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A121" t="s">
         <v>244</v>
       </c>
@@ -3767,7 +3818,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="122" spans="1:6" ht="48" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A122" t="s">
         <v>246</v>
       </c>
@@ -3781,27 +3832,27 @@
         <v>1</v>
       </c>
     </row>
-    <row r="123" spans="1:6" ht="224" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:8" ht="255" x14ac:dyDescent="0.25">
       <c r="A123" t="s">
         <v>248</v>
       </c>
-      <c r="B123" s="5" t="s">
+      <c r="B123" s="7" t="s">
         <v>249</v>
       </c>
-      <c r="C123" s="6" t="s">
+      <c r="C123" s="8" t="s">
         <v>410</v>
       </c>
-      <c r="D123" s="5" t="s">
-        <v>461</v>
-      </c>
-      <c r="E123" s="6" t="b">
+      <c r="D123" s="7" t="s">
+        <v>458</v>
+      </c>
+      <c r="E123" s="8" t="b">
         <v>1</v>
       </c>
       <c r="F123" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="124" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A124" t="s">
         <v>250</v>
       </c>
@@ -3815,27 +3866,27 @@
         <v>1</v>
       </c>
     </row>
-    <row r="125" spans="1:6" ht="112" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:8" ht="135" x14ac:dyDescent="0.25">
       <c r="A125" t="s">
         <v>252</v>
       </c>
-      <c r="B125" s="5" t="s">
+      <c r="B125" s="7" t="s">
         <v>253</v>
       </c>
-      <c r="C125" s="6" t="s">
+      <c r="C125" s="8" t="s">
         <v>410</v>
       </c>
-      <c r="D125" s="5" t="s">
-        <v>462</v>
-      </c>
-      <c r="E125" s="6" t="b">
+      <c r="D125" s="7" t="s">
+        <v>459</v>
+      </c>
+      <c r="E125" s="8" t="b">
         <v>1</v>
       </c>
       <c r="F125" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A126" t="s">
         <v>254</v>
       </c>
@@ -3849,27 +3900,27 @@
         <v>1</v>
       </c>
     </row>
-    <row r="127" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A127" t="s">
         <v>256</v>
       </c>
-      <c r="B127" s="5" t="s">
+      <c r="B127" s="7" t="s">
         <v>257</v>
       </c>
-      <c r="C127" s="6" t="s">
-        <v>409</v>
-      </c>
-      <c r="D127" s="5" t="s">
-        <v>463</v>
-      </c>
-      <c r="E127" s="6" t="b">
+      <c r="C127" s="8" t="s">
+        <v>408</v>
+      </c>
+      <c r="D127" s="7" t="s">
+        <v>480</v>
+      </c>
+      <c r="E127" s="8" t="b">
         <v>1</v>
       </c>
       <c r="F127" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="128" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A128" t="s">
         <v>258</v>
       </c>
@@ -3883,7 +3934,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="129" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A129" t="s">
         <v>260</v>
       </c>
@@ -3897,7 +3948,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="130" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A130" t="s">
         <v>262</v>
       </c>
@@ -3911,7 +3962,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="131" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A131" t="s">
         <v>264</v>
       </c>
@@ -3925,7 +3976,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="132" spans="1:6" ht="80" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:6" ht="90" x14ac:dyDescent="0.25">
       <c r="A132" t="s">
         <v>266</v>
       </c>
@@ -3939,7 +3990,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="133" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A133" t="s">
         <v>268</v>
       </c>
@@ -3953,7 +4004,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="134" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A134" t="s">
         <v>270</v>
       </c>
@@ -3967,7 +4018,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="135" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A135" t="s">
         <v>272</v>
       </c>
@@ -3981,7 +4032,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="136" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A136" t="s">
         <v>274</v>
       </c>
@@ -3995,7 +4046,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="137" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A137" t="s">
         <v>276</v>
       </c>
@@ -4009,7 +4060,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="138" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A138" t="s">
         <v>278</v>
       </c>
@@ -4023,7 +4074,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="139" spans="1:6" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A139" t="s">
         <v>280</v>
       </c>
@@ -4037,7 +4088,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="140" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A140" t="s">
         <v>282</v>
       </c>
@@ -4051,7 +4102,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="141" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A141" t="s">
         <v>284</v>
       </c>
@@ -4065,7 +4116,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="142" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A142" t="s">
         <v>286</v>
       </c>
@@ -4079,7 +4130,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="143" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A143" t="s">
         <v>288</v>
       </c>
@@ -4093,7 +4144,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="144" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A144" t="s">
         <v>290</v>
       </c>
@@ -4107,7 +4158,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="145" spans="1:6" ht="48" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A145" t="s">
         <v>292</v>
       </c>
@@ -4121,7 +4172,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="146" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A146" t="s">
         <v>294</v>
       </c>
@@ -4135,27 +4186,27 @@
         <v>1</v>
       </c>
     </row>
-    <row r="147" spans="1:6" ht="48" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A147" t="s">
         <v>296</v>
       </c>
-      <c r="B147" s="5" t="s">
+      <c r="B147" s="7" t="s">
         <v>297</v>
       </c>
-      <c r="C147" s="6" t="s">
+      <c r="C147" s="8" t="s">
         <v>409</v>
       </c>
-      <c r="D147" s="5" t="s">
-        <v>464</v>
-      </c>
-      <c r="E147" s="6" t="b">
+      <c r="D147" s="7" t="s">
+        <v>460</v>
+      </c>
+      <c r="E147" s="8" t="b">
         <v>1</v>
       </c>
       <c r="F147" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="148" spans="1:6" ht="96" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:6" ht="105" x14ac:dyDescent="0.25">
       <c r="A148" t="s">
         <v>298</v>
       </c>
@@ -4166,13 +4217,13 @@
         <v>412</v>
       </c>
       <c r="D148" s="3" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="F148" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="149" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A149" t="s">
         <v>300</v>
       </c>
@@ -4186,7 +4237,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="150" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A150" t="s">
         <v>302</v>
       </c>
@@ -4200,25 +4251,25 @@
         <v>1</v>
       </c>
     </row>
-    <row r="151" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A151" t="s">
         <v>304</v>
       </c>
-      <c r="B151" s="5" t="s">
+      <c r="B151" s="7" t="s">
         <v>305</v>
       </c>
-      <c r="C151" s="6" t="s">
-        <v>408</v>
-      </c>
-      <c r="D151" s="5"/>
-      <c r="E151" s="6" t="b">
+      <c r="C151" s="8" t="s">
+        <v>408</v>
+      </c>
+      <c r="D151" s="7"/>
+      <c r="E151" s="8" t="b">
         <v>1</v>
       </c>
       <c r="F151" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="152" spans="1:6" ht="128" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:6" ht="150" x14ac:dyDescent="0.25">
       <c r="A152" t="s">
         <v>306</v>
       </c>
@@ -4232,23 +4283,25 @@
         <v>0</v>
       </c>
     </row>
-    <row r="153" spans="1:6" ht="80" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:6" ht="90" x14ac:dyDescent="0.25">
       <c r="A153" t="s">
         <v>308</v>
       </c>
-      <c r="B153" s="5" t="s">
+      <c r="B153" s="7" t="s">
         <v>309</v>
       </c>
-      <c r="C153" s="6"/>
-      <c r="D153" s="5"/>
-      <c r="E153" s="6" t="b">
+      <c r="C153" s="8" t="s">
+        <v>411</v>
+      </c>
+      <c r="D153" s="7"/>
+      <c r="E153" s="8" t="b">
         <v>1</v>
       </c>
       <c r="F153" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="154" spans="1:6" ht="208" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:6" ht="225" x14ac:dyDescent="0.25">
       <c r="A154" t="s">
         <v>310</v>
       </c>
@@ -4262,7 +4315,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A155" t="s">
         <v>312</v>
       </c>
@@ -4276,515 +4329,721 @@
         <v>1</v>
       </c>
     </row>
-    <row r="156" spans="1:6" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A156" t="s">
         <v>314</v>
       </c>
       <c r="B156" s="3" t="s">
         <v>315</v>
       </c>
+      <c r="C156" t="s">
+        <v>408</v>
+      </c>
       <c r="F156" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="157" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A157" t="s">
         <v>316</v>
       </c>
       <c r="B157" s="3" t="s">
         <v>317</v>
       </c>
+      <c r="C157" t="s">
+        <v>408</v>
+      </c>
       <c r="F157" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="158" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A158" t="s">
         <v>318</v>
       </c>
       <c r="B158" s="3" t="s">
         <v>319</v>
       </c>
+      <c r="C158" t="s">
+        <v>408</v>
+      </c>
       <c r="F158" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="159" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A159" t="s">
         <v>320</v>
       </c>
       <c r="B159" s="3" t="s">
         <v>321</v>
       </c>
+      <c r="C159" t="s">
+        <v>408</v>
+      </c>
       <c r="F159" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="160" spans="1:6" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A160" t="s">
         <v>322</v>
       </c>
       <c r="B160" s="3" t="s">
         <v>323</v>
       </c>
+      <c r="C160" t="s">
+        <v>412</v>
+      </c>
       <c r="F160" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A161" t="s">
         <v>324</v>
       </c>
       <c r="B161" s="3" t="s">
         <v>325</v>
       </c>
+      <c r="C161" t="s">
+        <v>408</v>
+      </c>
       <c r="F161" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="162" spans="1:6" ht="96" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:6" ht="105" x14ac:dyDescent="0.25">
       <c r="A162" t="s">
         <v>326</v>
       </c>
-      <c r="B162" s="3" t="s">
+      <c r="B162" s="7" t="s">
         <v>327</v>
       </c>
+      <c r="C162" s="8" t="s">
+        <v>411</v>
+      </c>
+      <c r="D162" s="7" t="s">
+        <v>479</v>
+      </c>
+      <c r="E162" s="8" t="b">
+        <v>1</v>
+      </c>
       <c r="F162" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="163" spans="1:6" ht="256" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:6" ht="285" x14ac:dyDescent="0.25">
       <c r="A163" t="s">
         <v>328</v>
       </c>
       <c r="B163" s="3" t="s">
         <v>329</v>
       </c>
+      <c r="C163" t="s">
+        <v>412</v>
+      </c>
       <c r="F163" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="164" spans="1:6" ht="112" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:6" ht="120" x14ac:dyDescent="0.25">
       <c r="A164" t="s">
         <v>330</v>
       </c>
       <c r="B164" s="3" t="s">
         <v>331</v>
       </c>
+      <c r="C164" t="s">
+        <v>412</v>
+      </c>
       <c r="F164" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="165" spans="1:6" ht="176" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:6" ht="195" x14ac:dyDescent="0.25">
       <c r="A165" t="s">
         <v>332</v>
       </c>
-      <c r="B165" s="3" t="s">
+      <c r="B165" s="7" t="s">
         <v>333</v>
       </c>
+      <c r="C165" s="8" t="s">
+        <v>412</v>
+      </c>
+      <c r="D165" s="7" t="s">
+        <v>481</v>
+      </c>
+      <c r="E165" s="8"/>
       <c r="F165" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="166" spans="1:6" ht="192" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:6" ht="225" x14ac:dyDescent="0.25">
       <c r="A166" t="s">
         <v>334</v>
       </c>
       <c r="B166" s="3" t="s">
         <v>335</v>
       </c>
+      <c r="C166" t="s">
+        <v>412</v>
+      </c>
+      <c r="D166" s="3" t="s">
+        <v>461</v>
+      </c>
       <c r="F166" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="167" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A167" t="s">
         <v>336</v>
       </c>
       <c r="B167" s="3" t="s">
         <v>337</v>
       </c>
+      <c r="C167" t="s">
+        <v>408</v>
+      </c>
       <c r="F167" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="168" spans="1:6" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A168" t="s">
         <v>338</v>
       </c>
-      <c r="B168" s="3" t="s">
+      <c r="B168" s="7" t="s">
         <v>339</v>
       </c>
+      <c r="C168" s="8" t="s">
+        <v>410</v>
+      </c>
+      <c r="D168" s="7" t="s">
+        <v>462</v>
+      </c>
+      <c r="E168" s="8" t="b">
+        <v>1</v>
+      </c>
       <c r="F168" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="169" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A169" t="s">
         <v>340</v>
       </c>
       <c r="B169" s="3" t="s">
         <v>341</v>
       </c>
+      <c r="C169" t="s">
+        <v>408</v>
+      </c>
       <c r="F169" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="170" spans="1:6" ht="96" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:6" ht="105" x14ac:dyDescent="0.25">
       <c r="A170" t="s">
         <v>342</v>
       </c>
       <c r="B170" s="3" t="s">
         <v>343</v>
       </c>
+      <c r="C170" t="s">
+        <v>411</v>
+      </c>
       <c r="F170" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="171" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A171" t="s">
         <v>344</v>
       </c>
-      <c r="B171" s="3" t="s">
+      <c r="B171" s="7" t="s">
         <v>345</v>
       </c>
+      <c r="C171" s="8" t="s">
+        <v>408</v>
+      </c>
+      <c r="D171" s="7"/>
       <c r="F171" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="172" spans="1:6" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A172" t="s">
         <v>346</v>
       </c>
       <c r="B172" s="3" t="s">
         <v>347</v>
       </c>
+      <c r="C172" t="s">
+        <v>412</v>
+      </c>
+      <c r="D172" s="3" t="s">
+        <v>463</v>
+      </c>
       <c r="F172" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="173" spans="1:6" ht="304" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:6" ht="345" x14ac:dyDescent="0.25">
       <c r="A173" t="s">
         <v>348</v>
       </c>
       <c r="B173" s="3" t="s">
         <v>349</v>
       </c>
+      <c r="C173" t="s">
+        <v>411</v>
+      </c>
       <c r="F173" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="174" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A174" t="s">
         <v>350</v>
       </c>
       <c r="B174" s="3" t="s">
         <v>351</v>
       </c>
+      <c r="C174" t="s">
+        <v>408</v>
+      </c>
       <c r="F174" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="175" spans="1:6" ht="176" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:6" ht="195" x14ac:dyDescent="0.25">
       <c r="A175" t="s">
         <v>352</v>
       </c>
       <c r="B175" s="3" t="s">
         <v>353</v>
       </c>
+      <c r="C175" t="s">
+        <v>412</v>
+      </c>
+      <c r="D175" s="3" t="s">
+        <v>466</v>
+      </c>
       <c r="F175" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="176" spans="1:6" ht="96" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:6" ht="105" x14ac:dyDescent="0.25">
       <c r="A176" t="s">
         <v>354</v>
       </c>
       <c r="B176" s="3" t="s">
         <v>355</v>
       </c>
+      <c r="C176" t="s">
+        <v>407</v>
+      </c>
       <c r="F176" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="177" spans="1:6" ht="320" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:6" ht="345" x14ac:dyDescent="0.25">
       <c r="A177" t="s">
         <v>356</v>
       </c>
       <c r="B177" s="3" t="s">
         <v>357</v>
       </c>
+      <c r="C177" t="s">
+        <v>412</v>
+      </c>
       <c r="F177" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="178" spans="1:6" ht="144" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:6" ht="150" x14ac:dyDescent="0.25">
       <c r="A178" t="s">
         <v>358</v>
       </c>
       <c r="B178" s="3" t="s">
         <v>359</v>
       </c>
+      <c r="C178" t="s">
+        <v>408</v>
+      </c>
       <c r="F178" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="179" spans="1:6" ht="256" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:6" ht="300" x14ac:dyDescent="0.25">
       <c r="A179" t="s">
         <v>360</v>
       </c>
       <c r="B179" s="3" t="s">
         <v>361</v>
       </c>
+      <c r="C179" t="s">
+        <v>411</v>
+      </c>
+      <c r="D179" s="3" t="s">
+        <v>467</v>
+      </c>
       <c r="F179" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="180" spans="1:6" ht="208" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:6" ht="225" x14ac:dyDescent="0.25">
       <c r="A180" t="s">
         <v>362</v>
       </c>
       <c r="B180" s="3" t="s">
         <v>363</v>
       </c>
+      <c r="C180" t="s">
+        <v>412</v>
+      </c>
+      <c r="D180" s="3" t="s">
+        <v>468</v>
+      </c>
       <c r="F180" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="181" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A181" t="s">
         <v>364</v>
       </c>
       <c r="B181" s="3" t="s">
         <v>365</v>
       </c>
+      <c r="C181" t="s">
+        <v>408</v>
+      </c>
       <c r="F181" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="182" spans="1:6" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A182" t="s">
         <v>366</v>
       </c>
       <c r="B182" s="3" t="s">
         <v>367</v>
       </c>
+      <c r="C182" t="s">
+        <v>412</v>
+      </c>
       <c r="F182" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="183" spans="1:6" ht="96" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:6" ht="105" x14ac:dyDescent="0.25">
       <c r="A183" t="s">
         <v>368</v>
       </c>
       <c r="B183" s="3" t="s">
         <v>369</v>
       </c>
+      <c r="C183" t="s">
+        <v>412</v>
+      </c>
       <c r="F183" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="184" spans="1:6" ht="48" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:6" ht="45" x14ac:dyDescent="0.25">
       <c r="A184" t="s">
         <v>370</v>
       </c>
       <c r="B184" s="3" t="s">
         <v>371</v>
       </c>
+      <c r="C184" t="s">
+        <v>412</v>
+      </c>
       <c r="F184" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="185" spans="1:6" ht="144" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:6" ht="165" x14ac:dyDescent="0.25">
       <c r="A185" t="s">
         <v>372</v>
       </c>
       <c r="B185" s="3" t="s">
         <v>373</v>
       </c>
+      <c r="C185" t="s">
+        <v>410</v>
+      </c>
+      <c r="D185" s="3" t="s">
+        <v>469</v>
+      </c>
       <c r="F185" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="186" spans="1:6" ht="176" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:6" ht="195" x14ac:dyDescent="0.25">
       <c r="A186" t="s">
         <v>374</v>
       </c>
-      <c r="B186" s="3" t="s">
+      <c r="B186" s="7" t="s">
         <v>375</v>
       </c>
+      <c r="C186" s="8" t="s">
+        <v>410</v>
+      </c>
+      <c r="D186" s="7" t="s">
+        <v>470</v>
+      </c>
+      <c r="E186" s="8" t="b">
+        <v>1</v>
+      </c>
       <c r="F186" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="187" spans="1:6" ht="80" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:6" ht="90" x14ac:dyDescent="0.25">
       <c r="A187" t="s">
         <v>376</v>
       </c>
       <c r="B187" s="3" t="s">
         <v>377</v>
       </c>
+      <c r="C187" t="s">
+        <v>412</v>
+      </c>
       <c r="F187" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="188" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:6" ht="60" x14ac:dyDescent="0.25">
       <c r="A188" t="s">
         <v>378</v>
       </c>
-      <c r="B188" s="3" t="s">
+      <c r="B188" s="7" t="s">
         <v>379</v>
       </c>
+      <c r="C188" s="8" t="s">
+        <v>409</v>
+      </c>
+      <c r="D188" s="7" t="s">
+        <v>471</v>
+      </c>
+      <c r="E188" s="8" t="b">
+        <v>1</v>
+      </c>
       <c r="F188" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="189" spans="1:6" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A189" t="s">
         <v>380</v>
       </c>
       <c r="B189" s="3" t="s">
         <v>381</v>
       </c>
+      <c r="C189" t="s">
+        <v>412</v>
+      </c>
+      <c r="D189" s="3" t="s">
+        <v>472</v>
+      </c>
       <c r="F189" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="190" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A190" t="s">
         <v>382</v>
       </c>
       <c r="B190" s="3" t="s">
         <v>383</v>
       </c>
+      <c r="C190" t="s">
+        <v>408</v>
+      </c>
       <c r="F190" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="191" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A191" t="s">
         <v>384</v>
       </c>
       <c r="B191" s="3" t="s">
         <v>385</v>
       </c>
+      <c r="C191" t="s">
+        <v>408</v>
+      </c>
       <c r="F191" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="192" spans="1:6" ht="409.6" x14ac:dyDescent="0.2">
+    <row r="192" spans="1:6" ht="409.5" x14ac:dyDescent="0.25">
       <c r="A192" t="s">
         <v>386</v>
       </c>
       <c r="B192" s="3" t="s">
         <v>387</v>
       </c>
+      <c r="C192" t="s">
+        <v>412</v>
+      </c>
       <c r="F192" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="193" spans="1:6" ht="240" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:6" ht="270" x14ac:dyDescent="0.25">
       <c r="A193" t="s">
         <v>388</v>
       </c>
       <c r="B193" s="3" t="s">
         <v>389</v>
       </c>
+      <c r="C193" t="s">
+        <v>412</v>
+      </c>
+      <c r="D193" s="3" t="s">
+        <v>476</v>
+      </c>
       <c r="F193" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="194" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A194" t="s">
         <v>390</v>
       </c>
       <c r="B194" s="3" t="s">
         <v>391</v>
       </c>
+      <c r="C194" t="s">
+        <v>408</v>
+      </c>
       <c r="F194" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="195" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A195" t="s">
         <v>392</v>
       </c>
       <c r="B195" s="3" t="s">
         <v>393</v>
       </c>
+      <c r="C195" t="s">
+        <v>408</v>
+      </c>
       <c r="F195" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="196" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="196" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A196" t="s">
         <v>394</v>
       </c>
       <c r="B196" s="3" t="s">
         <v>395</v>
       </c>
+      <c r="C196" t="s">
+        <v>409</v>
+      </c>
+      <c r="D196" s="3" t="s">
+        <v>473</v>
+      </c>
       <c r="F196" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="197" spans="1:6" ht="224" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:6" ht="240" x14ac:dyDescent="0.25">
       <c r="A197" t="s">
         <v>396</v>
       </c>
-      <c r="B197" s="3" t="s">
+      <c r="B197" s="7" t="s">
         <v>397</v>
       </c>
+      <c r="C197" s="8" t="s">
+        <v>410</v>
+      </c>
+      <c r="D197" s="7" t="s">
+        <v>474</v>
+      </c>
+      <c r="E197" s="8" t="b">
+        <v>1</v>
+      </c>
       <c r="F197" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="198" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A198" t="s">
         <v>398</v>
       </c>
       <c r="B198" s="3" t="s">
         <v>399</v>
       </c>
+      <c r="C198" t="s">
+        <v>408</v>
+      </c>
       <c r="F198" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="199" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A199" t="s">
         <v>400</v>
       </c>
       <c r="B199" s="3" t="s">
         <v>401</v>
       </c>
+      <c r="C199" t="s">
+        <v>408</v>
+      </c>
       <c r="F199" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="200" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A200" t="s">
         <v>402</v>
       </c>
       <c r="B200" s="3" t="s">
         <v>403</v>
       </c>
+      <c r="C200" t="s">
+        <v>412</v>
+      </c>
+      <c r="D200" s="3" t="s">
+        <v>475</v>
+      </c>
+      <c r="E200" t="b">
+        <v>1</v>
+      </c>
       <c r="F200" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="201" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+    <row r="201" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A201" t="s">
         <v>404</v>
       </c>
       <c r="B201" s="3" t="s">
         <v>405</v>
       </c>
+      <c r="C201" t="s">
+        <v>408</v>
+      </c>
       <c r="F201" t="b">
         <v>1</v>
       </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C1:C83 C85:C145 C147:C1048576" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C1:C83 C85:C145 C147:C1048576">
       <formula1>$G$2:$G$7</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>